<commit_message>
updates custom table output
</commit_message>
<xml_diff>
--- a/data/processed/sam_auto_dashboard_2025_Q1/custom_table_output/bls_segment7_occ_highlights.xlsx
+++ b/data/processed/sam_auto_dashboard_2025_Q1/custom_table_output/bls_segment7_occ_highlights.xlsx
@@ -1417,7 +1417,7 @@
         <v>365.6</v>
       </c>
       <c r="N2" s="1">
-        <v>0</v>
+        <v>386.1732049325275</v>
       </c>
       <c r="O2" t="s">
         <v>35</v>
@@ -1479,7 +1479,7 @@
         <v>211.2</v>
       </c>
       <c r="N3" s="1">
-        <v>0</v>
+        <v>74.20554420607192</v>
       </c>
       <c r="O3" t="s">
         <v>36</v>
@@ -1538,7 +1538,7 @@
         <v>29.2</v>
       </c>
       <c r="N4" s="1">
-        <v>0</v>
+        <v>32.7958730628951</v>
       </c>
       <c r="O4" t="s">
         <v>35</v>
@@ -1600,7 +1600,7 @@
         <v>117</v>
       </c>
       <c r="N5" s="1">
-        <v>0</v>
+        <v>3.884940769227031</v>
       </c>
       <c r="O5" t="s">
         <v>36</v>
@@ -1656,7 +1656,7 @@
         <v>10.6</v>
       </c>
       <c r="N6" s="1">
-        <v>0</v>
+        <v>4.716466642874359</v>
       </c>
       <c r="O6" t="s">
         <v>35</v>
@@ -1715,7 +1715,7 @@
         <v>133.2</v>
       </c>
       <c r="N7" s="1">
-        <v>0</v>
+        <v>4.490634878002823</v>
       </c>
       <c r="O7" t="s">
         <v>36</v>
@@ -1860,7 +1860,7 @@
         <v>117</v>
       </c>
       <c r="N2" s="1">
-        <v>0</v>
+        <v>3.884940769227031</v>
       </c>
       <c r="O2" t="s">
         <v>36</v>
@@ -1916,7 +1916,7 @@
         <v>10.6</v>
       </c>
       <c r="N3" s="1">
-        <v>0</v>
+        <v>4.716466642874359</v>
       </c>
       <c r="O3" t="s">
         <v>35</v>
@@ -1975,7 +1975,7 @@
         <v>133.2</v>
       </c>
       <c r="N4" s="1">
-        <v>0</v>
+        <v>4.490634878002823</v>
       </c>
       <c r="O4" t="s">
         <v>36</v>
@@ -2037,7 +2037,7 @@
         <v>211.2</v>
       </c>
       <c r="N5" s="1">
-        <v>0</v>
+        <v>74.20554420607192</v>
       </c>
       <c r="O5" t="s">
         <v>36</v>
@@ -2096,7 +2096,7 @@
         <v>29.2</v>
       </c>
       <c r="N6" s="1">
-        <v>0</v>
+        <v>32.7958730628951</v>
       </c>
       <c r="O6" t="s">
         <v>35</v>
@@ -2158,7 +2158,7 @@
         <v>365.6</v>
       </c>
       <c r="N7" s="1">
-        <v>0</v>
+        <v>386.1732049325275</v>
       </c>
       <c r="O7" t="s">
         <v>35</v>
@@ -2303,7 +2303,7 @@
         <v>1406.7</v>
       </c>
       <c r="N2" s="1">
-        <v>0</v>
+        <v>6861.283954608292</v>
       </c>
       <c r="O2" t="s">
         <v>35</v>
@@ -2365,7 +2365,7 @@
         <v>115.2</v>
       </c>
       <c r="N3" s="1">
-        <v>0</v>
+        <v>922.4202957440928</v>
       </c>
       <c r="O3" t="s">
         <v>35</v>
@@ -2427,7 +2427,7 @@
         <v>14</v>
       </c>
       <c r="N4" s="1">
-        <v>0</v>
+        <v>253.3264998307637</v>
       </c>
       <c r="O4" t="s">
         <v>35</v>
@@ -2489,7 +2489,7 @@
         <v>37.6</v>
       </c>
       <c r="N5" s="1">
-        <v>0</v>
+        <v>333.5745409603368</v>
       </c>
       <c r="O5" t="s">
         <v>243</v>
@@ -2551,7 +2551,7 @@
         <v>559.2</v>
       </c>
       <c r="N6" s="1">
-        <v>0</v>
+        <v>516.9986322673582</v>
       </c>
       <c r="O6" t="s">
         <v>35</v>
@@ -2613,7 +2613,7 @@
         <v>609.3000000000001</v>
       </c>
       <c r="N7" s="1">
-        <v>0</v>
+        <v>471.1258262275985</v>
       </c>
       <c r="O7" t="s">
         <v>35</v>
@@ -2675,7 +2675,7 @@
         <v>3843</v>
       </c>
       <c r="N8" s="1">
-        <v>0</v>
+        <v>525.6239049259281</v>
       </c>
       <c r="O8" t="s">
         <v>244</v>
@@ -2737,7 +2737,7 @@
         <v>687.6</v>
       </c>
       <c r="N9" s="1">
-        <v>0</v>
+        <v>250.37449587335</v>
       </c>
       <c r="O9" t="s">
         <v>244</v>
@@ -2799,7 +2799,7 @@
         <v>265.5</v>
       </c>
       <c r="N10" s="1">
-        <v>0</v>
+        <v>240.3390775357394</v>
       </c>
       <c r="O10" t="s">
         <v>35</v>
@@ -2861,7 +2861,7 @@
         <v>127.2</v>
       </c>
       <c r="N11" s="1">
-        <v>0</v>
+        <v>207.8292216279649</v>
       </c>
       <c r="O11" t="s">
         <v>35</v>
@@ -2923,7 +2923,7 @@
         <v>693</v>
       </c>
       <c r="N12" s="1">
-        <v>0</v>
+        <v>149.8194801835526</v>
       </c>
       <c r="O12" t="s">
         <v>35</v>
@@ -2985,7 +2985,7 @@
         <v>19.2</v>
       </c>
       <c r="N13" s="1">
-        <v>0</v>
+        <v>184.7589182889105</v>
       </c>
       <c r="O13" t="s">
         <v>35</v>
@@ -3047,7 +3047,7 @@
         <v>136.8</v>
       </c>
       <c r="N14" s="1">
-        <v>0</v>
+        <v>234.3091776640756</v>
       </c>
       <c r="O14" t="s">
         <v>36</v>
@@ -3109,7 +3109,7 @@
         <v>201.6</v>
       </c>
       <c r="N15" s="1">
-        <v>0</v>
+        <v>387.2525226207051</v>
       </c>
       <c r="O15" t="s">
         <v>36</v>
@@ -3168,7 +3168,7 @@
         <v>89.60000000000001</v>
       </c>
       <c r="N16" s="1">
-        <v>0</v>
+        <v>248.4356548388555</v>
       </c>
       <c r="O16" t="s">
         <v>35</v>
@@ -3230,7 +3230,7 @@
         <v>50.4</v>
       </c>
       <c r="N17" s="1">
-        <v>0</v>
+        <v>128.4966051306644</v>
       </c>
       <c r="O17" t="s">
         <v>245</v>
@@ -3289,7 +3289,7 @@
         <v>177.6</v>
       </c>
       <c r="N18" s="1">
-        <v>0</v>
+        <v>140.3766571528158</v>
       </c>
       <c r="O18" t="s">
         <v>35</v>
@@ -3351,7 +3351,7 @@
         <v>272.8</v>
       </c>
       <c r="N19" s="1">
-        <v>0</v>
+        <v>104.6321499926035</v>
       </c>
       <c r="O19" t="s">
         <v>35</v>
@@ -3413,7 +3413,7 @@
         <v>648</v>
       </c>
       <c r="N20" s="1">
-        <v>0</v>
+        <v>307.105540245145</v>
       </c>
       <c r="O20" t="s">
         <v>35</v>
@@ -3475,7 +3475,7 @@
         <v>144.8</v>
       </c>
       <c r="N21" s="1">
-        <v>0</v>
+        <v>208.3982879751641</v>
       </c>
       <c r="O21" t="s">
         <v>36</v>
@@ -3534,7 +3534,7 @@
         <v>3.6</v>
       </c>
       <c r="N22" s="1">
-        <v>0</v>
+        <v>31.83433782712065</v>
       </c>
       <c r="O22" t="s">
         <v>35</v>
@@ -3596,7 +3596,7 @@
         <v>410.4</v>
       </c>
       <c r="N23" s="1">
-        <v>0</v>
+        <v>222.878410285862</v>
       </c>
       <c r="O23" t="s">
         <v>35</v>
@@ -3658,7 +3658,7 @@
         <v>116</v>
       </c>
       <c r="N24" s="1">
-        <v>0</v>
+        <v>90.6630193990094</v>
       </c>
       <c r="O24" t="s">
         <v>36</v>
@@ -3720,7 +3720,7 @@
         <v>1598</v>
       </c>
       <c r="N25" s="1">
-        <v>0</v>
+        <v>94.4718123952869</v>
       </c>
       <c r="O25" t="s">
         <v>35</v>
@@ -3782,7 +3782,7 @@
         <v>3087</v>
       </c>
       <c r="N26" s="1">
-        <v>0</v>
+        <v>79.09953304865576</v>
       </c>
       <c r="O26" t="s">
         <v>36</v>
@@ -3844,7 +3844,7 @@
         <v>108</v>
       </c>
       <c r="N27" s="1">
-        <v>0</v>
+        <v>36.09020464778688</v>
       </c>
       <c r="O27" t="s">
         <v>35</v>
@@ -3906,7 +3906,7 @@
         <v>2824</v>
       </c>
       <c r="N28" s="1">
-        <v>0</v>
+        <v>82.11893633265019</v>
       </c>
       <c r="O28" t="s">
         <v>35</v>
@@ -3968,7 +3968,7 @@
         <v>1700</v>
       </c>
       <c r="N29" s="1">
-        <v>0</v>
+        <v>56.90917102504978</v>
       </c>
       <c r="O29" t="s">
         <v>246</v>
@@ -4030,7 +4030,7 @@
         <v>33</v>
       </c>
       <c r="N30" s="1">
-        <v>0</v>
+        <v>35.80317334918507</v>
       </c>
       <c r="O30" t="s">
         <v>35</v>
@@ -4092,7 +4092,7 @@
         <v>818</v>
       </c>
       <c r="N31" s="1">
-        <v>0</v>
+        <v>74.49584127135387</v>
       </c>
       <c r="O31" t="s">
         <v>36</v>
@@ -4151,7 +4151,7 @@
         <v>524</v>
       </c>
       <c r="N32" s="1">
-        <v>0</v>
+        <v>72.49981043935509</v>
       </c>
       <c r="O32" t="s">
         <v>35</v>
@@ -4213,7 +4213,7 @@
         <v>15.6</v>
       </c>
       <c r="N33" s="1">
-        <v>0</v>
+        <v>36.84683321106351</v>
       </c>
       <c r="O33" t="s">
         <v>35</v>
@@ -4275,7 +4275,7 @@
         <v>118</v>
       </c>
       <c r="N34" s="1">
-        <v>0</v>
+        <v>58.69041087703511</v>
       </c>
       <c r="O34" t="s">
         <v>35</v>
@@ -4337,7 +4337,7 @@
         <v>469.8</v>
       </c>
       <c r="N35" s="1">
-        <v>0</v>
+        <v>101.8869347047059</v>
       </c>
       <c r="O35" t="s">
         <v>36</v>
@@ -4399,7 +4399,7 @@
         <v>22.4</v>
       </c>
       <c r="N36" s="1">
-        <v>0</v>
+        <v>52.56865584596185</v>
       </c>
       <c r="O36" t="s">
         <v>245</v>
@@ -4458,7 +4458,7 @@
         <v>1242</v>
       </c>
       <c r="N37" s="1">
-        <v>0</v>
+        <v>49.81580339270992</v>
       </c>
       <c r="O37" t="s">
         <v>36</v>
@@ -4517,7 +4517,7 @@
         <v>317.1</v>
       </c>
       <c r="N38" s="1">
-        <v>0</v>
+        <v>39.89348983754204</v>
       </c>
       <c r="O38" t="s">
         <v>35</v>
@@ -4579,7 +4579,7 @@
         <v>1148</v>
       </c>
       <c r="N39" s="1">
-        <v>0</v>
+        <v>69.19683453679401</v>
       </c>
       <c r="O39" t="s">
         <v>35</v>
@@ -4641,7 +4641,7 @@
         <v>4723</v>
       </c>
       <c r="N40" s="1">
-        <v>0</v>
+        <v>95.28846510115214</v>
       </c>
       <c r="O40" t="s">
         <v>244</v>
@@ -4703,7 +4703,7 @@
         <v>2.4</v>
       </c>
       <c r="N41" s="1">
-        <v>0</v>
+        <v>15.18058663539603</v>
       </c>
       <c r="O41" t="s">
         <v>244</v>
@@ -4765,7 +4765,7 @@
         <v>1445</v>
       </c>
       <c r="N42" s="1">
-        <v>0</v>
+        <v>33.63271709201708</v>
       </c>
       <c r="O42" t="s">
         <v>35</v>
@@ -4827,7 +4827,7 @@
         <v>3417</v>
       </c>
       <c r="N43" s="1">
-        <v>0</v>
+        <v>42.84307302105591</v>
       </c>
       <c r="O43" t="s">
         <v>35</v>
@@ -4889,7 +4889,7 @@
         <v>757.4</v>
       </c>
       <c r="N44" s="1">
-        <v>0</v>
+        <v>42.1406087983756</v>
       </c>
       <c r="O44" t="s">
         <v>36</v>
@@ -4948,7 +4948,7 @@
         <v>3513</v>
       </c>
       <c r="N45" s="1">
-        <v>0</v>
+        <v>62.32890934486505</v>
       </c>
       <c r="O45" t="s">
         <v>244</v>
@@ -5010,7 +5010,7 @@
         <v>189.6</v>
       </c>
       <c r="N46" s="1">
-        <v>0</v>
+        <v>40.02223498224424</v>
       </c>
       <c r="O46" t="s">
         <v>35</v>
@@ -5072,7 +5072,7 @@
         <v>79.19999999999999</v>
       </c>
       <c r="N47" s="1">
-        <v>0</v>
+        <v>39.97390454866906</v>
       </c>
       <c r="O47" t="s">
         <v>36</v>
@@ -5134,7 +5134,7 @@
         <v>11</v>
       </c>
       <c r="N48" s="1">
-        <v>0</v>
+        <v>4.877372865551081</v>
       </c>
       <c r="O48" t="s">
         <v>35</v>
@@ -5196,7 +5196,7 @@
         <v>14.4</v>
       </c>
       <c r="N49" s="1">
-        <v>0</v>
+        <v>110.5187139612092</v>
       </c>
       <c r="O49" t="s">
         <v>35</v>
@@ -5258,7 +5258,7 @@
         <v>35</v>
       </c>
       <c r="N50" s="1">
-        <v>0</v>
+        <v>14.70392847993301</v>
       </c>
       <c r="O50" t="s">
         <v>36</v>
@@ -5320,7 +5320,7 @@
         <v>408</v>
       </c>
       <c r="N51" s="1">
-        <v>0</v>
+        <v>14.12382153621653</v>
       </c>
       <c r="O51" t="s">
         <v>246</v>
@@ -5382,7 +5382,7 @@
         <v>161.1</v>
       </c>
       <c r="N52" s="1">
-        <v>0</v>
+        <v>22.50712780800693</v>
       </c>
       <c r="O52" t="s">
         <v>36</v>
@@ -5444,7 +5444,7 @@
         <v>703.8000000000001</v>
       </c>
       <c r="N53" s="1">
-        <v>0</v>
+        <v>57.52353890923705</v>
       </c>
       <c r="O53" t="s">
         <v>36</v>
@@ -5503,7 +5503,7 @@
         <v>490</v>
       </c>
       <c r="N54" s="1">
-        <v>0</v>
+        <v>42.73331147173693</v>
       </c>
       <c r="O54" t="s">
         <v>36</v>
@@ -5565,7 +5565,7 @@
         <v>7.5</v>
       </c>
       <c r="N55" s="1">
-        <v>0</v>
+        <v>12.15260944481739</v>
       </c>
       <c r="O55" t="s">
         <v>35</v>
@@ -5627,7 +5627,7 @@
         <v>370</v>
       </c>
       <c r="N56" s="1">
-        <v>0</v>
+        <v>30.63158816206036</v>
       </c>
       <c r="O56" t="s">
         <v>244</v>
@@ -5689,7 +5689,7 @@
         <v>51.2</v>
       </c>
       <c r="N57" s="1">
-        <v>0</v>
+        <v>24.46215824850296</v>
       </c>
       <c r="O57" t="s">
         <v>36</v>
@@ -5751,7 +5751,7 @@
         <v>2028</v>
       </c>
       <c r="N58" s="1">
-        <v>0</v>
+        <v>27.06582596638111</v>
       </c>
       <c r="O58" t="s">
         <v>35</v>
@@ -5813,7 +5813,7 @@
         <v>142.2</v>
       </c>
       <c r="N59" s="1">
-        <v>0</v>
+        <v>83.42707445865703</v>
       </c>
       <c r="O59" t="s">
         <v>35</v>
@@ -5875,7 +5875,7 @@
         <v>205.2</v>
       </c>
       <c r="N60" s="1">
-        <v>0</v>
+        <v>18.58576019079173</v>
       </c>
       <c r="O60" t="s">
         <v>36</v>
@@ -5934,7 +5934,7 @@
         <v>143</v>
       </c>
       <c r="N61" s="1">
-        <v>0</v>
+        <v>6.719535260243862</v>
       </c>
       <c r="O61" t="s">
         <v>36</v>
@@ -5993,7 +5993,7 @@
         <v>81.89999999999999</v>
       </c>
       <c r="N62" s="1">
-        <v>0</v>
+        <v>20.19270496073999</v>
       </c>
       <c r="O62" t="s">
         <v>36</v>
@@ -6052,7 +6052,7 @@
         <v>7.6</v>
       </c>
       <c r="N63" s="1">
-        <v>0</v>
+        <v>15.96951254840345</v>
       </c>
       <c r="O63" t="s">
         <v>35</v>
@@ -6111,7 +6111,7 @@
         <v>175.7</v>
       </c>
       <c r="N64" s="1">
-        <v>0</v>
+        <v>23.98791767505791</v>
       </c>
       <c r="O64" t="s">
         <v>36</v>
@@ -6170,7 +6170,7 @@
         <v>6</v>
       </c>
       <c r="N65" s="1">
-        <v>0</v>
+        <v>9.085647648466988</v>
       </c>
       <c r="O65" t="s">
         <v>35</v>
@@ -6232,7 +6232,7 @@
         <v>42.4</v>
       </c>
       <c r="N66" s="1">
-        <v>0</v>
+        <v>8.35126428294145</v>
       </c>
       <c r="O66" t="s">
         <v>245</v>
@@ -6288,7 +6288,7 @@
         <v>65.10000000000001</v>
       </c>
       <c r="N67" s="1">
-        <v>0</v>
+        <v>18.23429176317842</v>
       </c>
       <c r="O67" t="s">
         <v>36</v>
@@ -6347,7 +6347,7 @@
         <v>483</v>
       </c>
       <c r="N68" s="1">
-        <v>0</v>
+        <v>15.77784856608914</v>
       </c>
       <c r="O68" t="s">
         <v>35</v>
@@ -6409,7 +6409,7 @@
         <v>2138.4</v>
       </c>
       <c r="N69" s="1">
-        <v>0</v>
+        <v>33.7807946476311</v>
       </c>
       <c r="O69" t="s">
         <v>243</v>
@@ -6471,7 +6471,7 @@
         <v>50.40000000000001</v>
       </c>
       <c r="N70" s="1">
-        <v>0</v>
+        <v>14.4821181545651</v>
       </c>
       <c r="O70" t="s">
         <v>245</v>
@@ -6530,7 +6530,7 @@
         <v>23.6</v>
       </c>
       <c r="N71" s="1">
-        <v>0</v>
+        <v>10.1393048335376</v>
       </c>
       <c r="O71" t="s">
         <v>35</v>
@@ -6589,7 +6589,7 @@
         <v>155.4</v>
       </c>
       <c r="N72" s="1">
-        <v>0</v>
+        <v>8.035449173674619</v>
       </c>
       <c r="O72" t="s">
         <v>36</v>
@@ -6651,7 +6651,7 @@
         <v>746</v>
       </c>
       <c r="N73" s="1">
-        <v>0</v>
+        <v>39.63622270594832</v>
       </c>
       <c r="O73" t="s">
         <v>36</v>
@@ -6713,7 +6713,7 @@
         <v>551.6999999999999</v>
       </c>
       <c r="N74" s="1">
-        <v>0</v>
+        <v>17.88233177571537</v>
       </c>
       <c r="O74" t="s">
         <v>35</v>
@@ -6775,7 +6775,7 @@
         <v>4.5</v>
       </c>
       <c r="N75" s="1">
-        <v>0</v>
+        <v>4.698010824388477</v>
       </c>
       <c r="O75" t="s">
         <v>36</v>
@@ -6834,7 +6834,7 @@
         <v>26.4</v>
       </c>
       <c r="N76" s="1">
-        <v>0</v>
+        <v>9.854643729556518</v>
       </c>
       <c r="O76" t="s">
         <v>245</v>
@@ -6893,7 +6893,7 @@
         <v>4.4</v>
       </c>
       <c r="N77" s="1">
-        <v>0</v>
+        <v>4.096231117553382</v>
       </c>
       <c r="O77" t="s">
         <v>35</v>
@@ -6955,7 +6955,7 @@
         <v>9.4</v>
       </c>
       <c r="N78" s="1">
-        <v>0</v>
+        <v>10.31192652085174</v>
       </c>
       <c r="O78" t="s">
         <v>244</v>
@@ -7017,7 +7017,7 @@
         <v>22.8</v>
       </c>
       <c r="N79" s="1">
-        <v>0</v>
+        <v>12.09351633128016</v>
       </c>
       <c r="O79" t="s">
         <v>36</v>
@@ -7076,7 +7076,7 @@
         <v>280</v>
       </c>
       <c r="N80" s="1">
-        <v>0</v>
+        <v>20.28554497550737</v>
       </c>
       <c r="O80" t="s">
         <v>243</v>
@@ -7138,7 +7138,7 @@
         <v>351.2</v>
       </c>
       <c r="N81" s="1">
-        <v>0</v>
+        <v>19.31609516060931</v>
       </c>
       <c r="O81" t="s">
         <v>36</v>
@@ -7200,7 +7200,7 @@
         <v>10</v>
       </c>
       <c r="N82" s="1">
-        <v>0</v>
+        <v>5.645628489968562</v>
       </c>
       <c r="O82" t="s">
         <v>35</v>
@@ -7262,7 +7262,7 @@
         <v>686.6999999999999</v>
       </c>
       <c r="N83" s="1">
-        <v>0</v>
+        <v>15.83093927041445</v>
       </c>
       <c r="O83" t="s">
         <v>36</v>
@@ -7324,7 +7324,7 @@
         <v>1.3</v>
       </c>
       <c r="N84" s="1">
-        <v>0</v>
+        <v>7.411073055449902</v>
       </c>
       <c r="O84" t="s">
         <v>245</v>
@@ -7383,7 +7383,7 @@
         <v>27</v>
       </c>
       <c r="N85" s="1">
-        <v>0</v>
+        <v>8.411512027490273</v>
       </c>
       <c r="O85" t="s">
         <v>245</v>
@@ -7442,7 +7442,7 @@
         <v>132</v>
       </c>
       <c r="N86" s="1">
-        <v>0</v>
+        <v>73.18186678178051</v>
       </c>
       <c r="O86" t="s">
         <v>35</v>
@@ -7504,7 +7504,7 @@
         <v>24</v>
       </c>
       <c r="N87" s="1">
-        <v>0</v>
+        <v>5.649213015993937</v>
       </c>
       <c r="O87" t="s">
         <v>35</v>
@@ -7566,7 +7566,7 @@
         <v>3.8</v>
       </c>
       <c r="N88" s="1">
-        <v>0</v>
+        <v>7.53578155291019</v>
       </c>
       <c r="O88" t="s">
         <v>35</v>
@@ -7625,7 +7625,7 @@
         <v>21.7</v>
       </c>
       <c r="N89" s="1">
-        <v>0</v>
+        <v>12.76351470660874</v>
       </c>
       <c r="O89" t="s">
         <v>243</v>
@@ -7687,7 +7687,7 @@
         <v>872</v>
       </c>
       <c r="N90" s="1">
-        <v>0</v>
+        <v>17.93764447325695</v>
       </c>
       <c r="O90" t="s">
         <v>36</v>
@@ -7746,7 +7746,7 @@
         <v>148</v>
       </c>
       <c r="N91" s="1">
-        <v>0</v>
+        <v>13.42953312578718</v>
       </c>
       <c r="O91" t="s">
         <v>35</v>
@@ -7808,7 +7808,7 @@
         <v>74.40000000000001</v>
       </c>
       <c r="N92" s="1">
-        <v>0</v>
+        <v>4.432866838487374</v>
       </c>
       <c r="O92" t="s">
         <v>35</v>
@@ -7870,7 +7870,7 @@
         <v>8.5</v>
       </c>
       <c r="N93" s="1">
-        <v>0</v>
+        <v>4.999335683176739</v>
       </c>
       <c r="O93" t="s">
         <v>35</v>
@@ -7929,7 +7929,7 @@
         <v>190.4</v>
       </c>
       <c r="N94" s="1">
-        <v>0</v>
+        <v>5.083461083498125</v>
       </c>
       <c r="O94" t="s">
         <v>36</v>
@@ -7991,7 +7991,7 @@
         <v>65</v>
       </c>
       <c r="N95" s="1">
-        <v>0</v>
+        <v>5.036083056079515</v>
       </c>
       <c r="O95" t="s">
         <v>35</v>
@@ -8053,7 +8053,7 @@
         <v>240.1</v>
       </c>
       <c r="N96" s="1">
-        <v>0</v>
+        <v>7.778839321565147</v>
       </c>
       <c r="O96" t="s">
         <v>36</v>
@@ -8115,7 +8115,7 @@
         <v>6</v>
       </c>
       <c r="N97" s="1">
-        <v>0</v>
+        <v>5.441696998756923</v>
       </c>
       <c r="O97" t="s">
         <v>36</v>
@@ -8174,7 +8174,7 @@
         <v>921.6</v>
       </c>
       <c r="N98" s="1">
-        <v>0</v>
+        <v>84.72706744014472</v>
       </c>
       <c r="O98" t="s">
         <v>36</v>
@@ -8233,7 +8233,7 @@
         <v>20.5</v>
       </c>
       <c r="N99" s="1">
-        <v>0</v>
+        <v>3.164817210882059</v>
       </c>
       <c r="O99" t="s">
         <v>35</v>
@@ -8292,7 +8292,7 @@
         <v>52</v>
       </c>
       <c r="N100" s="1">
-        <v>0</v>
+        <v>4.224273047748467</v>
       </c>
       <c r="O100" t="s">
         <v>244</v>
@@ -8354,7 +8354,7 @@
         <v>74.09999999999999</v>
       </c>
       <c r="N101" s="1">
-        <v>0</v>
+        <v>5.763286156288465</v>
       </c>
       <c r="O101" t="s">
         <v>35</v>
@@ -8499,7 +8499,7 @@
         <v>11</v>
       </c>
       <c r="N2" s="1">
-        <v>0</v>
+        <v>4.877372865551081</v>
       </c>
       <c r="O2" t="s">
         <v>35</v>
@@ -8561,7 +8561,7 @@
         <v>4.4</v>
       </c>
       <c r="N3" s="1">
-        <v>0</v>
+        <v>4.096231117553382</v>
       </c>
       <c r="O3" t="s">
         <v>35</v>
@@ -8623,7 +8623,7 @@
         <v>42.4</v>
       </c>
       <c r="N4" s="1">
-        <v>0</v>
+        <v>8.35126428294145</v>
       </c>
       <c r="O4" t="s">
         <v>245</v>
@@ -8679,7 +8679,7 @@
         <v>3.6</v>
       </c>
       <c r="N5" s="1">
-        <v>0</v>
+        <v>31.83433782712065</v>
       </c>
       <c r="O5" t="s">
         <v>35</v>
@@ -8741,7 +8741,7 @@
         <v>7.5</v>
       </c>
       <c r="N6" s="1">
-        <v>0</v>
+        <v>12.15260944481739</v>
       </c>
       <c r="O6" t="s">
         <v>35</v>
@@ -8803,7 +8803,7 @@
         <v>4.5</v>
       </c>
       <c r="N7" s="1">
-        <v>0</v>
+        <v>4.698010824388477</v>
       </c>
       <c r="O7" t="s">
         <v>36</v>
@@ -8862,7 +8862,7 @@
         <v>35</v>
       </c>
       <c r="N8" s="1">
-        <v>0</v>
+        <v>14.70392847993301</v>
       </c>
       <c r="O8" t="s">
         <v>36</v>
@@ -8924,7 +8924,7 @@
         <v>23.6</v>
       </c>
       <c r="N9" s="1">
-        <v>0</v>
+        <v>10.1393048335376</v>
       </c>
       <c r="O9" t="s">
         <v>35</v>
@@ -8983,7 +8983,7 @@
         <v>2.4</v>
       </c>
       <c r="N10" s="1">
-        <v>0</v>
+        <v>15.18058663539603</v>
       </c>
       <c r="O10" t="s">
         <v>244</v>
@@ -9045,7 +9045,7 @@
         <v>6</v>
       </c>
       <c r="N11" s="1">
-        <v>0</v>
+        <v>9.085647648466988</v>
       </c>
       <c r="O11" t="s">
         <v>35</v>
@@ -9107,7 +9107,7 @@
         <v>14</v>
       </c>
       <c r="N12" s="1">
-        <v>0</v>
+        <v>253.3264998307637</v>
       </c>
       <c r="O12" t="s">
         <v>35</v>
@@ -9169,7 +9169,7 @@
         <v>10</v>
       </c>
       <c r="N13" s="1">
-        <v>0</v>
+        <v>5.645628489968562</v>
       </c>
       <c r="O13" t="s">
         <v>35</v>
@@ -9231,7 +9231,7 @@
         <v>108</v>
       </c>
       <c r="N14" s="1">
-        <v>0</v>
+        <v>36.09020464778688</v>
       </c>
       <c r="O14" t="s">
         <v>35</v>
@@ -9293,7 +9293,7 @@
         <v>20.5</v>
       </c>
       <c r="N15" s="1">
-        <v>0</v>
+        <v>3.164817210882059</v>
       </c>
       <c r="O15" t="s">
         <v>35</v>
@@ -9352,7 +9352,7 @@
         <v>143</v>
       </c>
       <c r="N16" s="1">
-        <v>0</v>
+        <v>6.719535260243862</v>
       </c>
       <c r="O16" t="s">
         <v>36</v>
@@ -9411,7 +9411,7 @@
         <v>52</v>
       </c>
       <c r="N17" s="1">
-        <v>0</v>
+        <v>4.224273047748467</v>
       </c>
       <c r="O17" t="s">
         <v>244</v>
@@ -9473,7 +9473,7 @@
         <v>24</v>
       </c>
       <c r="N18" s="1">
-        <v>0</v>
+        <v>5.649213015993937</v>
       </c>
       <c r="O18" t="s">
         <v>35</v>
@@ -9535,7 +9535,7 @@
         <v>3.8</v>
       </c>
       <c r="N19" s="1">
-        <v>0</v>
+        <v>7.53578155291019</v>
       </c>
       <c r="O19" t="s">
         <v>35</v>
@@ -9594,7 +9594,7 @@
         <v>155.4</v>
       </c>
       <c r="N20" s="1">
-        <v>0</v>
+        <v>8.035449173674619</v>
       </c>
       <c r="O20" t="s">
         <v>36</v>
@@ -9656,7 +9656,7 @@
         <v>9.4</v>
       </c>
       <c r="N21" s="1">
-        <v>0</v>
+        <v>10.31192652085174</v>
       </c>
       <c r="O21" t="s">
         <v>244</v>
@@ -9718,7 +9718,7 @@
         <v>483</v>
       </c>
       <c r="N22" s="1">
-        <v>0</v>
+        <v>15.77784856608914</v>
       </c>
       <c r="O22" t="s">
         <v>35</v>
@@ -9780,7 +9780,7 @@
         <v>115.2</v>
       </c>
       <c r="N23" s="1">
-        <v>0</v>
+        <v>922.4202957440928</v>
       </c>
       <c r="O23" t="s">
         <v>35</v>
@@ -9842,7 +9842,7 @@
         <v>37.6</v>
       </c>
       <c r="N24" s="1">
-        <v>0</v>
+        <v>333.5745409603368</v>
       </c>
       <c r="O24" t="s">
         <v>243</v>
@@ -9904,7 +9904,7 @@
         <v>127.2</v>
       </c>
       <c r="N25" s="1">
-        <v>0</v>
+        <v>207.8292216279649</v>
       </c>
       <c r="O25" t="s">
         <v>35</v>
@@ -9966,7 +9966,7 @@
         <v>693</v>
       </c>
       <c r="N26" s="1">
-        <v>0</v>
+        <v>149.8194801835526</v>
       </c>
       <c r="O26" t="s">
         <v>35</v>
@@ -10028,7 +10028,7 @@
         <v>33</v>
       </c>
       <c r="N27" s="1">
-        <v>0</v>
+        <v>35.80317334918507</v>
       </c>
       <c r="O27" t="s">
         <v>35</v>
@@ -10090,7 +10090,7 @@
         <v>408</v>
       </c>
       <c r="N28" s="1">
-        <v>0</v>
+        <v>14.12382153621653</v>
       </c>
       <c r="O28" t="s">
         <v>246</v>
@@ -10152,7 +10152,7 @@
         <v>15.6</v>
       </c>
       <c r="N29" s="1">
-        <v>0</v>
+        <v>36.84683321106351</v>
       </c>
       <c r="O29" t="s">
         <v>35</v>
@@ -10214,7 +10214,7 @@
         <v>317.1</v>
       </c>
       <c r="N30" s="1">
-        <v>0</v>
+        <v>39.89348983754204</v>
       </c>
       <c r="O30" t="s">
         <v>35</v>
@@ -10276,7 +10276,7 @@
         <v>118</v>
       </c>
       <c r="N31" s="1">
-        <v>0</v>
+        <v>58.69041087703511</v>
       </c>
       <c r="O31" t="s">
         <v>35</v>
@@ -10338,7 +10338,7 @@
         <v>1700</v>
       </c>
       <c r="N32" s="1">
-        <v>0</v>
+        <v>56.90917102504978</v>
       </c>
       <c r="O32" t="s">
         <v>246</v>
@@ -10400,7 +10400,7 @@
         <v>7.6</v>
       </c>
       <c r="N33" s="1">
-        <v>0</v>
+        <v>15.96951254840345</v>
       </c>
       <c r="O33" t="s">
         <v>35</v>
@@ -10459,7 +10459,7 @@
         <v>8.5</v>
       </c>
       <c r="N34" s="1">
-        <v>0</v>
+        <v>4.999335683176739</v>
       </c>
       <c r="O34" t="s">
         <v>35</v>
@@ -10518,7 +10518,7 @@
         <v>65</v>
       </c>
       <c r="N35" s="1">
-        <v>0</v>
+        <v>5.036083056079515</v>
       </c>
       <c r="O35" t="s">
         <v>35</v>
@@ -10580,7 +10580,7 @@
         <v>190.4</v>
       </c>
       <c r="N36" s="1">
-        <v>0</v>
+        <v>5.083461083498125</v>
       </c>
       <c r="O36" t="s">
         <v>36</v>
@@ -10642,7 +10642,7 @@
         <v>74.40000000000001</v>
       </c>
       <c r="N37" s="1">
-        <v>0</v>
+        <v>4.432866838487374</v>
       </c>
       <c r="O37" t="s">
         <v>35</v>
@@ -10704,7 +10704,7 @@
         <v>1.3</v>
       </c>
       <c r="N38" s="1">
-        <v>0</v>
+        <v>7.411073055449902</v>
       </c>
       <c r="O38" t="s">
         <v>245</v>
@@ -10763,7 +10763,7 @@
         <v>27</v>
       </c>
       <c r="N39" s="1">
-        <v>0</v>
+        <v>8.411512027490273</v>
       </c>
       <c r="O39" t="s">
         <v>245</v>
@@ -10822,7 +10822,7 @@
         <v>185.6</v>
       </c>
       <c r="N40" s="1">
-        <v>0</v>
+        <v>3.187988318213764</v>
       </c>
       <c r="O40" t="s">
         <v>36</v>
@@ -10884,7 +10884,7 @@
         <v>26.4</v>
       </c>
       <c r="N41" s="1">
-        <v>0</v>
+        <v>9.854643729556518</v>
       </c>
       <c r="O41" t="s">
         <v>245</v>
@@ -10943,7 +10943,7 @@
         <v>265.5</v>
       </c>
       <c r="N42" s="1">
-        <v>0</v>
+        <v>240.3390775357394</v>
       </c>
       <c r="O42" t="s">
         <v>35</v>
@@ -11005,7 +11005,7 @@
         <v>3417</v>
       </c>
       <c r="N43" s="1">
-        <v>0</v>
+        <v>42.84307302105591</v>
       </c>
       <c r="O43" t="s">
         <v>35</v>
@@ -11067,7 +11067,7 @@
         <v>370</v>
       </c>
       <c r="N44" s="1">
-        <v>0</v>
+        <v>30.63158816206036</v>
       </c>
       <c r="O44" t="s">
         <v>244</v>
@@ -11129,7 +11129,7 @@
         <v>19.2</v>
       </c>
       <c r="N45" s="1">
-        <v>0</v>
+        <v>184.7589182889105</v>
       </c>
       <c r="O45" t="s">
         <v>35</v>
@@ -11191,7 +11191,7 @@
         <v>161.1</v>
       </c>
       <c r="N46" s="1">
-        <v>0</v>
+        <v>22.50712780800693</v>
       </c>
       <c r="O46" t="s">
         <v>36</v>
@@ -11253,7 +11253,7 @@
         <v>177.6</v>
       </c>
       <c r="N47" s="1">
-        <v>0</v>
+        <v>140.3766571528158</v>
       </c>
       <c r="O47" t="s">
         <v>35</v>
@@ -11315,7 +11315,7 @@
         <v>687.6</v>
       </c>
       <c r="N48" s="1">
-        <v>0</v>
+        <v>250.37449587335</v>
       </c>
       <c r="O48" t="s">
         <v>244</v>
@@ -11377,7 +11377,7 @@
         <v>50.40000000000001</v>
       </c>
       <c r="N49" s="1">
-        <v>0</v>
+        <v>14.4821181545651</v>
       </c>
       <c r="O49" t="s">
         <v>245</v>
@@ -11436,7 +11436,7 @@
         <v>1445</v>
       </c>
       <c r="N50" s="1">
-        <v>0</v>
+        <v>33.63271709201708</v>
       </c>
       <c r="O50" t="s">
         <v>35</v>
@@ -11498,7 +11498,7 @@
         <v>272.8</v>
       </c>
       <c r="N51" s="1">
-        <v>0</v>
+        <v>104.6321499926035</v>
       </c>
       <c r="O51" t="s">
         <v>35</v>
@@ -11560,7 +11560,7 @@
         <v>189.6</v>
       </c>
       <c r="N52" s="1">
-        <v>0</v>
+        <v>40.02223498224424</v>
       </c>
       <c r="O52" t="s">
         <v>35</v>
@@ -11622,7 +11622,7 @@
         <v>2028</v>
       </c>
       <c r="N53" s="1">
-        <v>0</v>
+        <v>27.06582596638111</v>
       </c>
       <c r="O53" t="s">
         <v>35</v>
@@ -11684,7 +11684,7 @@
         <v>2824</v>
       </c>
       <c r="N54" s="1">
-        <v>0</v>
+        <v>82.11893633265019</v>
       </c>
       <c r="O54" t="s">
         <v>35</v>
@@ -11746,7 +11746,7 @@
         <v>50.4</v>
       </c>
       <c r="N55" s="1">
-        <v>0</v>
+        <v>128.4966051306644</v>
       </c>
       <c r="O55" t="s">
         <v>245</v>
@@ -11805,7 +11805,7 @@
         <v>559.2</v>
       </c>
       <c r="N56" s="1">
-        <v>0</v>
+        <v>516.9986322673582</v>
       </c>
       <c r="O56" t="s">
         <v>35</v>
@@ -11867,7 +11867,7 @@
         <v>961.6</v>
       </c>
       <c r="N57" s="1">
-        <v>0</v>
+        <v>5.119157635505013</v>
       </c>
       <c r="O57" t="s">
         <v>35</v>
@@ -11926,7 +11926,7 @@
         <v>551.6999999999999</v>
       </c>
       <c r="N58" s="1">
-        <v>0</v>
+        <v>17.88233177571537</v>
       </c>
       <c r="O58" t="s">
         <v>35</v>
@@ -11988,7 +11988,7 @@
         <v>3513</v>
       </c>
       <c r="N59" s="1">
-        <v>0</v>
+        <v>62.32890934486505</v>
       </c>
       <c r="O59" t="s">
         <v>244</v>
@@ -12050,7 +12050,7 @@
         <v>1598</v>
       </c>
       <c r="N60" s="1">
-        <v>0</v>
+        <v>94.4718123952869</v>
       </c>
       <c r="O60" t="s">
         <v>35</v>
@@ -12112,7 +12112,7 @@
         <v>51.2</v>
       </c>
       <c r="N61" s="1">
-        <v>0</v>
+        <v>24.46215824850296</v>
       </c>
       <c r="O61" t="s">
         <v>36</v>
@@ -12174,7 +12174,7 @@
         <v>3843</v>
       </c>
       <c r="N62" s="1">
-        <v>0</v>
+        <v>525.6239049259281</v>
       </c>
       <c r="O62" t="s">
         <v>244</v>
@@ -12236,7 +12236,7 @@
         <v>6</v>
       </c>
       <c r="N63" s="1">
-        <v>0</v>
+        <v>5.441696998756923</v>
       </c>
       <c r="O63" t="s">
         <v>36</v>
@@ -12295,7 +12295,7 @@
         <v>205.2</v>
       </c>
       <c r="N64" s="1">
-        <v>0</v>
+        <v>18.58576019079173</v>
       </c>
       <c r="O64" t="s">
         <v>36</v>
@@ -12354,7 +12354,7 @@
         <v>79.19999999999999</v>
       </c>
       <c r="N65" s="1">
-        <v>0</v>
+        <v>39.97390454866906</v>
       </c>
       <c r="O65" t="s">
         <v>36</v>
@@ -12416,7 +12416,7 @@
         <v>757.4</v>
       </c>
       <c r="N66" s="1">
-        <v>0</v>
+        <v>42.1406087983756</v>
       </c>
       <c r="O66" t="s">
         <v>36</v>
@@ -12475,7 +12475,7 @@
         <v>3087</v>
       </c>
       <c r="N67" s="1">
-        <v>0</v>
+        <v>79.09953304865576</v>
       </c>
       <c r="O67" t="s">
         <v>36</v>
@@ -12537,7 +12537,7 @@
         <v>22.4</v>
       </c>
       <c r="N68" s="1">
-        <v>0</v>
+        <v>52.56865584596185</v>
       </c>
       <c r="O68" t="s">
         <v>245</v>
@@ -12596,7 +12596,7 @@
         <v>609.3000000000001</v>
       </c>
       <c r="N69" s="1">
-        <v>0</v>
+        <v>471.1258262275985</v>
       </c>
       <c r="O69" t="s">
         <v>35</v>
@@ -12658,7 +12658,7 @@
         <v>21.7</v>
       </c>
       <c r="N70" s="1">
-        <v>0</v>
+        <v>12.76351470660874</v>
       </c>
       <c r="O70" t="s">
         <v>243</v>
@@ -12720,7 +12720,7 @@
         <v>1242</v>
       </c>
       <c r="N71" s="1">
-        <v>0</v>
+        <v>49.81580339270992</v>
       </c>
       <c r="O71" t="s">
         <v>36</v>
@@ -12779,7 +12779,7 @@
         <v>240.1</v>
       </c>
       <c r="N72" s="1">
-        <v>0</v>
+        <v>7.778839321565147</v>
       </c>
       <c r="O72" t="s">
         <v>36</v>
@@ -12841,7 +12841,7 @@
         <v>4723</v>
       </c>
       <c r="N73" s="1">
-        <v>0</v>
+        <v>95.28846510115214</v>
       </c>
       <c r="O73" t="s">
         <v>244</v>
@@ -12903,7 +12903,7 @@
         <v>818</v>
       </c>
       <c r="N74" s="1">
-        <v>0</v>
+        <v>74.49584127135387</v>
       </c>
       <c r="O74" t="s">
         <v>36</v>
@@ -12962,7 +12962,7 @@
         <v>136.8</v>
       </c>
       <c r="N75" s="1">
-        <v>0</v>
+        <v>234.3091776640756</v>
       </c>
       <c r="O75" t="s">
         <v>36</v>
@@ -13024,7 +13024,7 @@
         <v>81.89999999999999</v>
       </c>
       <c r="N76" s="1">
-        <v>0</v>
+        <v>20.19270496073999</v>
       </c>
       <c r="O76" t="s">
         <v>36</v>
@@ -13083,7 +13083,7 @@
         <v>524</v>
       </c>
       <c r="N77" s="1">
-        <v>0</v>
+        <v>72.49981043935509</v>
       </c>
       <c r="O77" t="s">
         <v>35</v>
@@ -13145,7 +13145,7 @@
         <v>93.90000000000001</v>
       </c>
       <c r="N78" s="1">
-        <v>0</v>
+        <v>3.036991043139647</v>
       </c>
       <c r="O78" t="s">
         <v>36</v>
@@ -13204,7 +13204,7 @@
         <v>22.8</v>
       </c>
       <c r="N79" s="1">
-        <v>0</v>
+        <v>12.09351633128016</v>
       </c>
       <c r="O79" t="s">
         <v>36</v>
@@ -13263,7 +13263,7 @@
         <v>74.09999999999999</v>
       </c>
       <c r="N80" s="1">
-        <v>0</v>
+        <v>5.763286156288465</v>
       </c>
       <c r="O80" t="s">
         <v>35</v>
@@ -13325,7 +13325,7 @@
         <v>2.2</v>
       </c>
       <c r="N81" s="1">
-        <v>0</v>
+        <v>2.796360442916767</v>
       </c>
       <c r="O81" t="s">
         <v>35</v>
@@ -13387,7 +13387,7 @@
         <v>65.10000000000001</v>
       </c>
       <c r="N82" s="1">
-        <v>0</v>
+        <v>18.23429176317842</v>
       </c>
       <c r="O82" t="s">
         <v>36</v>
@@ -13446,7 +13446,7 @@
         <v>116</v>
       </c>
       <c r="N83" s="1">
-        <v>0</v>
+        <v>90.6630193990094</v>
       </c>
       <c r="O83" t="s">
         <v>36</v>
@@ -13508,7 +13508,7 @@
         <v>175.7</v>
       </c>
       <c r="N84" s="1">
-        <v>0</v>
+        <v>23.98791767505791</v>
       </c>
       <c r="O84" t="s">
         <v>36</v>
@@ -13567,7 +13567,7 @@
         <v>686.6999999999999</v>
       </c>
       <c r="N85" s="1">
-        <v>0</v>
+        <v>15.83093927041445</v>
       </c>
       <c r="O85" t="s">
         <v>36</v>
@@ -13629,7 +13629,7 @@
         <v>89.60000000000001</v>
       </c>
       <c r="N86" s="1">
-        <v>0</v>
+        <v>248.4356548388555</v>
       </c>
       <c r="O86" t="s">
         <v>35</v>
@@ -13691,7 +13691,7 @@
         <v>1148</v>
       </c>
       <c r="N87" s="1">
-        <v>0</v>
+        <v>69.19683453679401</v>
       </c>
       <c r="O87" t="s">
         <v>35</v>
@@ -13753,7 +13753,7 @@
         <v>2138.4</v>
       </c>
       <c r="N88" s="1">
-        <v>0</v>
+        <v>33.7807946476311</v>
       </c>
       <c r="O88" t="s">
         <v>243</v>
@@ -13815,7 +13815,7 @@
         <v>490</v>
       </c>
       <c r="N89" s="1">
-        <v>0</v>
+        <v>42.73331147173693</v>
       </c>
       <c r="O89" t="s">
         <v>36</v>
@@ -13877,7 +13877,7 @@
         <v>351.2</v>
       </c>
       <c r="N90" s="1">
-        <v>0</v>
+        <v>19.31609516060931</v>
       </c>
       <c r="O90" t="s">
         <v>36</v>
@@ -13939,7 +13939,7 @@
         <v>280</v>
       </c>
       <c r="N91" s="1">
-        <v>0</v>
+        <v>20.28554497550737</v>
       </c>
       <c r="O91" t="s">
         <v>243</v>
@@ -14001,7 +14001,7 @@
         <v>469.8</v>
       </c>
       <c r="N92" s="1">
-        <v>0</v>
+        <v>101.8869347047059</v>
       </c>
       <c r="O92" t="s">
         <v>36</v>
@@ -14063,7 +14063,7 @@
         <v>148</v>
       </c>
       <c r="N93" s="1">
-        <v>0</v>
+        <v>13.42953312578718</v>
       </c>
       <c r="O93" t="s">
         <v>35</v>
@@ -14125,7 +14125,7 @@
         <v>1406.7</v>
       </c>
       <c r="N94" s="1">
-        <v>0</v>
+        <v>6861.283954608292</v>
       </c>
       <c r="O94" t="s">
         <v>35</v>
@@ -14187,7 +14187,7 @@
         <v>872</v>
       </c>
       <c r="N95" s="1">
-        <v>0</v>
+        <v>17.93764447325695</v>
       </c>
       <c r="O95" t="s">
         <v>36</v>
@@ -14246,7 +14246,7 @@
         <v>703.8000000000001</v>
       </c>
       <c r="N96" s="1">
-        <v>0</v>
+        <v>57.52353890923705</v>
       </c>
       <c r="O96" t="s">
         <v>36</v>
@@ -14305,7 +14305,7 @@
         <v>410.4</v>
       </c>
       <c r="N97" s="1">
-        <v>0</v>
+        <v>222.878410285862</v>
       </c>
       <c r="O97" t="s">
         <v>35</v>
@@ -14367,7 +14367,7 @@
         <v>648</v>
       </c>
       <c r="N98" s="1">
-        <v>0</v>
+        <v>307.105540245145</v>
       </c>
       <c r="O98" t="s">
         <v>35</v>
@@ -14429,7 +14429,7 @@
         <v>201.6</v>
       </c>
       <c r="N99" s="1">
-        <v>0</v>
+        <v>387.2525226207051</v>
       </c>
       <c r="O99" t="s">
         <v>36</v>
@@ -14488,7 +14488,7 @@
         <v>746</v>
       </c>
       <c r="N100" s="1">
-        <v>0</v>
+        <v>39.63622270594832</v>
       </c>
       <c r="O100" t="s">
         <v>36</v>
@@ -14550,7 +14550,7 @@
         <v>144.8</v>
       </c>
       <c r="N101" s="1">
-        <v>0</v>
+        <v>208.3982879751641</v>
       </c>
       <c r="O101" t="s">
         <v>36</v>
@@ -14692,7 +14692,7 @@
         <v>410.4</v>
       </c>
       <c r="N2" s="1">
-        <v>0</v>
+        <v>222.878410285862</v>
       </c>
       <c r="O2" t="s">
         <v>35</v>
@@ -14754,7 +14754,7 @@
         <v>142.2</v>
       </c>
       <c r="N3" s="1">
-        <v>0</v>
+        <v>83.42707445865703</v>
       </c>
       <c r="O3" t="s">
         <v>35</v>
@@ -14816,7 +14816,7 @@
         <v>89.60000000000001</v>
       </c>
       <c r="N4" s="1">
-        <v>0</v>
+        <v>248.4356548388555</v>
       </c>
       <c r="O4" t="s">
         <v>35</v>
@@ -14878,7 +14878,7 @@
         <v>609.3000000000001</v>
       </c>
       <c r="N5" s="1">
-        <v>0</v>
+        <v>471.1258262275985</v>
       </c>
       <c r="O5" t="s">
         <v>35</v>
@@ -14940,7 +14940,7 @@
         <v>108</v>
       </c>
       <c r="N6" s="1">
-        <v>0</v>
+        <v>36.09020464778688</v>
       </c>
       <c r="O6" t="s">
         <v>35</v>
@@ -15002,7 +15002,7 @@
         <v>29.2</v>
       </c>
       <c r="N7" s="1">
-        <v>0</v>
+        <v>32.7958730628951</v>
       </c>
       <c r="O7" t="s">
         <v>35</v>
@@ -15064,7 +15064,7 @@
         <v>1598</v>
       </c>
       <c r="N8" s="1">
-        <v>0</v>
+        <v>94.4718123952869</v>
       </c>
       <c r="O8" t="s">
         <v>35</v>
@@ -15126,7 +15126,7 @@
         <v>189.6</v>
       </c>
       <c r="N9" s="1">
-        <v>0</v>
+        <v>40.02223498224424</v>
       </c>
       <c r="O9" t="s">
         <v>35</v>
@@ -15188,7 +15188,7 @@
         <v>177.6</v>
       </c>
       <c r="N10" s="1">
-        <v>0</v>
+        <v>140.3766571528158</v>
       </c>
       <c r="O10" t="s">
         <v>35</v>
@@ -15250,7 +15250,7 @@
         <v>559.2</v>
       </c>
       <c r="N11" s="1">
-        <v>0</v>
+        <v>516.9986322673582</v>
       </c>
       <c r="O11" t="s">
         <v>35</v>
@@ -15312,7 +15312,7 @@
         <v>1148</v>
       </c>
       <c r="N12" s="1">
-        <v>0</v>
+        <v>69.19683453679401</v>
       </c>
       <c r="O12" t="s">
         <v>35</v>
@@ -15374,7 +15374,7 @@
         <v>132.5</v>
       </c>
       <c r="N13" s="1">
-        <v>0</v>
+        <v>3.900953436672769</v>
       </c>
       <c r="O13" t="s">
         <v>35</v>
@@ -15436,7 +15436,7 @@
         <v>4723</v>
       </c>
       <c r="N14" s="1">
-        <v>0</v>
+        <v>95.28846510115214</v>
       </c>
       <c r="O14" t="s">
         <v>244</v>
@@ -15498,7 +15498,7 @@
         <v>280</v>
       </c>
       <c r="N15" s="1">
-        <v>0</v>
+        <v>20.28554497550737</v>
       </c>
       <c r="O15" t="s">
         <v>243</v>
@@ -15560,7 +15560,7 @@
         <v>3417</v>
       </c>
       <c r="N16" s="1">
-        <v>0</v>
+        <v>42.84307302105591</v>
       </c>
       <c r="O16" t="s">
         <v>35</v>
@@ -15622,7 +15622,7 @@
         <v>3087</v>
       </c>
       <c r="N17" s="1">
-        <v>0</v>
+        <v>79.09953304865576</v>
       </c>
       <c r="O17" t="s">
         <v>36</v>
@@ -15684,7 +15684,7 @@
         <v>118</v>
       </c>
       <c r="N18" s="1">
-        <v>0</v>
+        <v>58.69041087703511</v>
       </c>
       <c r="O18" t="s">
         <v>35</v>
@@ -15746,7 +15746,7 @@
         <v>272.8</v>
       </c>
       <c r="N19" s="1">
-        <v>0</v>
+        <v>104.6321499926035</v>
       </c>
       <c r="O19" t="s">
         <v>35</v>
@@ -15808,7 +15808,7 @@
         <v>52</v>
       </c>
       <c r="N20" s="1">
-        <v>0</v>
+        <v>4.224273047748467</v>
       </c>
       <c r="O20" t="s">
         <v>244</v>
@@ -15870,7 +15870,7 @@
         <v>133.2</v>
       </c>
       <c r="N21" s="1">
-        <v>0</v>
+        <v>4.490634878002823</v>
       </c>
       <c r="O21" t="s">
         <v>36</v>
@@ -15932,7 +15932,7 @@
         <v>3843</v>
       </c>
       <c r="N22" s="1">
-        <v>0</v>
+        <v>525.6239049259281</v>
       </c>
       <c r="O22" t="s">
         <v>244</v>
@@ -15994,7 +15994,7 @@
         <v>351.2</v>
       </c>
       <c r="N23" s="1">
-        <v>0</v>
+        <v>19.31609516060931</v>
       </c>
       <c r="O23" t="s">
         <v>36</v>
@@ -16056,7 +16056,7 @@
         <v>28</v>
       </c>
       <c r="N24" s="1">
-        <v>0</v>
+        <v>4.410947131822462</v>
       </c>
       <c r="O24" t="s">
         <v>36</v>
@@ -16112,7 +16112,7 @@
         <v>24</v>
       </c>
       <c r="N25" s="1">
-        <v>0</v>
+        <v>5.649213015993937</v>
       </c>
       <c r="O25" t="s">
         <v>35</v>
@@ -16174,7 +16174,7 @@
         <v>10.6</v>
       </c>
       <c r="N26" s="1">
-        <v>0</v>
+        <v>4.716466642874359</v>
       </c>
       <c r="O26" t="s">
         <v>35</v>
@@ -16233,7 +16233,7 @@
         <v>469.8</v>
       </c>
       <c r="N27" s="1">
-        <v>0</v>
+        <v>101.8869347047059</v>
       </c>
       <c r="O27" t="s">
         <v>36</v>
@@ -16295,7 +16295,7 @@
         <v>551.6999999999999</v>
       </c>
       <c r="N28" s="1">
-        <v>0</v>
+        <v>17.88233177571537</v>
       </c>
       <c r="O28" t="s">
         <v>35</v>
@@ -16357,7 +16357,7 @@
         <v>211.2</v>
       </c>
       <c r="N29" s="1">
-        <v>0</v>
+        <v>74.20554420607192</v>
       </c>
       <c r="O29" t="s">
         <v>36</v>
@@ -16416,7 +16416,7 @@
         <v>21.7</v>
       </c>
       <c r="N30" s="1">
-        <v>0</v>
+        <v>12.76351470660874</v>
       </c>
       <c r="O30" t="s">
         <v>243</v>
@@ -16478,7 +16478,7 @@
         <v>2.2</v>
       </c>
       <c r="N31" s="1">
-        <v>0</v>
+        <v>2.796360442916767</v>
       </c>
       <c r="O31" t="s">
         <v>35</v>
@@ -16540,7 +16540,7 @@
         <v>853.6</v>
       </c>
       <c r="N32" s="1">
-        <v>0</v>
+        <v>8.205439441347828</v>
       </c>
       <c r="O32" t="s">
         <v>36</v>
@@ -16602,7 +16602,7 @@
         <v>148</v>
       </c>
       <c r="N33" s="1">
-        <v>0</v>
+        <v>13.42953312578718</v>
       </c>
       <c r="O33" t="s">
         <v>35</v>
@@ -16664,7 +16664,7 @@
         <v>1445</v>
       </c>
       <c r="N34" s="1">
-        <v>0</v>
+        <v>33.63271709201708</v>
       </c>
       <c r="O34" t="s">
         <v>35</v>
@@ -16726,7 +16726,7 @@
         <v>20.5</v>
       </c>
       <c r="N35" s="1">
-        <v>0</v>
+        <v>3.164817210882059</v>
       </c>
       <c r="O35" t="s">
         <v>35</v>
@@ -16785,7 +16785,7 @@
         <v>2028</v>
       </c>
       <c r="N36" s="1">
-        <v>0</v>
+        <v>27.06582596638111</v>
       </c>
       <c r="O36" t="s">
         <v>35</v>
@@ -16847,7 +16847,7 @@
         <v>93.90000000000001</v>
       </c>
       <c r="N37" s="1">
-        <v>0</v>
+        <v>3.036991043139647</v>
       </c>
       <c r="O37" t="s">
         <v>36</v>
@@ -16906,7 +16906,7 @@
         <v>693</v>
       </c>
       <c r="N38" s="1">
-        <v>0</v>
+        <v>149.8194801835526</v>
       </c>
       <c r="O38" t="s">
         <v>35</v>
@@ -16968,7 +16968,7 @@
         <v>872</v>
       </c>
       <c r="N39" s="1">
-        <v>0</v>
+        <v>17.93764447325695</v>
       </c>
       <c r="O39" t="s">
         <v>36</v>
@@ -17027,7 +17027,7 @@
         <v>33</v>
       </c>
       <c r="N40" s="1">
-        <v>0</v>
+        <v>35.80317334918507</v>
       </c>
       <c r="O40" t="s">
         <v>35</v>
@@ -17089,7 +17089,7 @@
         <v>74.09999999999999</v>
       </c>
       <c r="N41" s="1">
-        <v>0</v>
+        <v>5.763286156288465</v>
       </c>
       <c r="O41" t="s">
         <v>35</v>
@@ -17151,7 +17151,7 @@
         <v>10</v>
       </c>
       <c r="N42" s="1">
-        <v>0</v>
+        <v>5.645628489968562</v>
       </c>
       <c r="O42" t="s">
         <v>35</v>
@@ -17213,7 +17213,7 @@
         <v>2138.4</v>
       </c>
       <c r="N43" s="1">
-        <v>0</v>
+        <v>33.7807946476311</v>
       </c>
       <c r="O43" t="s">
         <v>243</v>
@@ -17275,7 +17275,7 @@
         <v>370</v>
       </c>
       <c r="N44" s="1">
-        <v>0</v>
+        <v>30.63158816206036</v>
       </c>
       <c r="O44" t="s">
         <v>244</v>
@@ -17337,7 +17337,7 @@
         <v>117</v>
       </c>
       <c r="N45" s="1">
-        <v>0</v>
+        <v>3.884940769227031</v>
       </c>
       <c r="O45" t="s">
         <v>36</v>
@@ -17393,7 +17393,7 @@
         <v>961.6</v>
       </c>
       <c r="N46" s="1">
-        <v>0</v>
+        <v>5.119157635505013</v>
       </c>
       <c r="O46" t="s">
         <v>35</v>
@@ -17452,7 +17452,7 @@
         <v>500.4</v>
       </c>
       <c r="N47" s="1">
-        <v>0</v>
+        <v>21.41117833339402</v>
       </c>
       <c r="O47" t="s">
         <v>36</v>
@@ -17514,7 +17514,7 @@
         <v>240.1</v>
       </c>
       <c r="N48" s="1">
-        <v>0</v>
+        <v>7.778839321565147</v>
       </c>
       <c r="O48" t="s">
         <v>36</v>
@@ -17576,7 +17576,7 @@
         <v>1242</v>
       </c>
       <c r="N49" s="1">
-        <v>0</v>
+        <v>49.81580339270992</v>
       </c>
       <c r="O49" t="s">
         <v>36</v>
@@ -17635,7 +17635,7 @@
         <v>6</v>
       </c>
       <c r="N50" s="1">
-        <v>0</v>
+        <v>5.441696998756923</v>
       </c>
       <c r="O50" t="s">
         <v>36</v>
@@ -17694,7 +17694,7 @@
         <v>818</v>
       </c>
       <c r="N51" s="1">
-        <v>0</v>
+        <v>74.49584127135387</v>
       </c>
       <c r="O51" t="s">
         <v>36</v>
@@ -17753,7 +17753,7 @@
         <v>2824</v>
       </c>
       <c r="N52" s="1">
-        <v>0</v>
+        <v>82.11893633265019</v>
       </c>
       <c r="O52" t="s">
         <v>35</v>
@@ -17815,7 +17815,7 @@
         <v>921.6</v>
       </c>
       <c r="N53" s="1">
-        <v>0</v>
+        <v>84.72706744014472</v>
       </c>
       <c r="O53" t="s">
         <v>36</v>
@@ -17874,7 +17874,7 @@
         <v>185.6</v>
       </c>
       <c r="N54" s="1">
-        <v>0</v>
+        <v>3.187988318213764</v>
       </c>
       <c r="O54" t="s">
         <v>36</v>
@@ -17936,7 +17936,7 @@
         <v>350</v>
       </c>
       <c r="N55" s="1">
-        <v>0</v>
+        <v>7.644018814864816</v>
       </c>
       <c r="O55" t="s">
         <v>35</v>
@@ -17998,7 +17998,7 @@
         <v>757.4</v>
       </c>
       <c r="N56" s="1">
-        <v>0</v>
+        <v>42.1406087983756</v>
       </c>
       <c r="O56" t="s">
         <v>36</v>
@@ -18057,7 +18057,7 @@
         <v>65.10000000000001</v>
       </c>
       <c r="N57" s="1">
-        <v>0</v>
+        <v>18.23429176317842</v>
       </c>
       <c r="O57" t="s">
         <v>36</v>
@@ -18116,7 +18116,7 @@
         <v>26.4</v>
       </c>
       <c r="N58" s="1">
-        <v>0</v>
+        <v>9.854643729556518</v>
       </c>
       <c r="O58" t="s">
         <v>245</v>
@@ -18175,7 +18175,7 @@
         <v>55.2</v>
       </c>
       <c r="N59" s="1">
-        <v>0</v>
+        <v>3.253820945677159</v>
       </c>
       <c r="O59" t="s">
         <v>36</v>
@@ -18231,7 +18231,7 @@
         <v>94.5</v>
       </c>
       <c r="N60" s="1">
-        <v>0</v>
+        <v>1.360706788473817</v>
       </c>
       <c r="O60" t="s">
         <v>278</v>
@@ -18290,7 +18290,7 @@
         <v>8.5</v>
       </c>
       <c r="N61" s="1">
-        <v>0</v>
+        <v>4.999335683176739</v>
       </c>
       <c r="O61" t="s">
         <v>35</v>
@@ -18349,7 +18349,7 @@
         <v>65</v>
       </c>
       <c r="N62" s="1">
-        <v>0</v>
+        <v>5.036083056079515</v>
       </c>
       <c r="O62" t="s">
         <v>35</v>
@@ -18411,7 +18411,7 @@
         <v>190.4</v>
       </c>
       <c r="N63" s="1">
-        <v>0</v>
+        <v>5.083461083498125</v>
       </c>
       <c r="O63" t="s">
         <v>36</v>
@@ -18473,7 +18473,7 @@
         <v>74.40000000000001</v>
       </c>
       <c r="N64" s="1">
-        <v>0</v>
+        <v>4.432866838487374</v>
       </c>
       <c r="O64" t="s">
         <v>35</v>
@@ -18535,7 +18535,7 @@
         <v>143</v>
       </c>
       <c r="N65" s="1">
-        <v>0</v>
+        <v>6.719535260243862</v>
       </c>
       <c r="O65" t="s">
         <v>36</v>
@@ -18594,7 +18594,7 @@
         <v>32.09999999999999</v>
       </c>
       <c r="N66" s="1">
-        <v>0</v>
+        <v>2.388843150352038</v>
       </c>
       <c r="O66" t="s">
         <v>35</v>
@@ -18653,7 +18653,7 @@
         <v>80.2</v>
       </c>
       <c r="N67" s="1">
-        <v>0</v>
+        <v>2.591989037920724</v>
       </c>
       <c r="O67" t="s">
         <v>243</v>
@@ -18715,7 +18715,7 @@
         <v>408</v>
       </c>
       <c r="N68" s="1">
-        <v>0</v>
+        <v>14.12382153621653</v>
       </c>
       <c r="O68" t="s">
         <v>246</v>
@@ -18777,7 +18777,7 @@
         <v>6</v>
       </c>
       <c r="N69" s="1">
-        <v>0</v>
+        <v>9.085647648466988</v>
       </c>
       <c r="O69" t="s">
         <v>35</v>
@@ -18839,7 +18839,7 @@
         <v>50.40000000000001</v>
       </c>
       <c r="N70" s="1">
-        <v>0</v>
+        <v>14.4821181545651</v>
       </c>
       <c r="O70" t="s">
         <v>245</v>
@@ -18898,7 +18898,7 @@
         <v>686.6999999999999</v>
       </c>
       <c r="N71" s="1">
-        <v>0</v>
+        <v>15.83093927041445</v>
       </c>
       <c r="O71" t="s">
         <v>36</v>
@@ -19043,7 +19043,7 @@
         <v>115.2</v>
       </c>
       <c r="N2" s="1">
-        <v>0</v>
+        <v>922.4202957440928</v>
       </c>
       <c r="O2" t="s">
         <v>35</v>
@@ -19105,7 +19105,7 @@
         <v>1406.7</v>
       </c>
       <c r="N3" s="1">
-        <v>0</v>
+        <v>6861.283954608292</v>
       </c>
       <c r="O3" t="s">
         <v>35</v>
@@ -19167,7 +19167,7 @@
         <v>37.6</v>
       </c>
       <c r="N4" s="1">
-        <v>0</v>
+        <v>333.5745409603368</v>
       </c>
       <c r="O4" t="s">
         <v>243</v>
@@ -19229,7 +19229,7 @@
         <v>648</v>
       </c>
       <c r="N5" s="1">
-        <v>0</v>
+        <v>307.105540245145</v>
       </c>
       <c r="O5" t="s">
         <v>35</v>
@@ -19291,7 +19291,7 @@
         <v>201.6</v>
       </c>
       <c r="N6" s="1">
-        <v>0</v>
+        <v>387.2525226207051</v>
       </c>
       <c r="O6" t="s">
         <v>36</v>
@@ -19350,7 +19350,7 @@
         <v>136.8</v>
       </c>
       <c r="N7" s="1">
-        <v>0</v>
+        <v>234.3091776640756</v>
       </c>
       <c r="O7" t="s">
         <v>36</v>
@@ -19412,7 +19412,7 @@
         <v>144.8</v>
       </c>
       <c r="N8" s="1">
-        <v>0</v>
+        <v>208.3982879751641</v>
       </c>
       <c r="O8" t="s">
         <v>36</v>
@@ -19471,7 +19471,7 @@
         <v>687.6</v>
       </c>
       <c r="N9" s="1">
-        <v>0</v>
+        <v>250.37449587335</v>
       </c>
       <c r="O9" t="s">
         <v>244</v>
@@ -19533,7 +19533,7 @@
         <v>19.2</v>
       </c>
       <c r="N10" s="1">
-        <v>0</v>
+        <v>184.7589182889105</v>
       </c>
       <c r="O10" t="s">
         <v>35</v>
@@ -19595,7 +19595,7 @@
         <v>14</v>
       </c>
       <c r="N11" s="1">
-        <v>0</v>
+        <v>253.3264998307637</v>
       </c>
       <c r="O11" t="s">
         <v>35</v>
@@ -19657,7 +19657,7 @@
         <v>14.4</v>
       </c>
       <c r="N12" s="1">
-        <v>0</v>
+        <v>110.5187139612092</v>
       </c>
       <c r="O12" t="s">
         <v>35</v>
@@ -19719,7 +19719,7 @@
         <v>127.2</v>
       </c>
       <c r="N13" s="1">
-        <v>0</v>
+        <v>207.8292216279649</v>
       </c>
       <c r="O13" t="s">
         <v>35</v>
@@ -19781,7 +19781,7 @@
         <v>265.5</v>
       </c>
       <c r="N14" s="1">
-        <v>0</v>
+        <v>240.3390775357394</v>
       </c>
       <c r="O14" t="s">
         <v>35</v>
@@ -19843,7 +19843,7 @@
         <v>116</v>
       </c>
       <c r="N15" s="1">
-        <v>0</v>
+        <v>90.6630193990094</v>
       </c>
       <c r="O15" t="s">
         <v>36</v>
@@ -19905,7 +19905,7 @@
         <v>365.6</v>
       </c>
       <c r="N16" s="1">
-        <v>0</v>
+        <v>386.1732049325275</v>
       </c>
       <c r="O16" t="s">
         <v>35</v>
@@ -19967,7 +19967,7 @@
         <v>3.6</v>
       </c>
       <c r="N17" s="1">
-        <v>0</v>
+        <v>31.83433782712065</v>
       </c>
       <c r="O17" t="s">
         <v>35</v>
@@ -20029,7 +20029,7 @@
         <v>132</v>
       </c>
       <c r="N18" s="1">
-        <v>0</v>
+        <v>73.18186678178051</v>
       </c>
       <c r="O18" t="s">
         <v>35</v>
@@ -20091,7 +20091,7 @@
         <v>50.4</v>
       </c>
       <c r="N19" s="1">
-        <v>0</v>
+        <v>128.4966051306644</v>
       </c>
       <c r="O19" t="s">
         <v>245</v>
@@ -20150,7 +20150,7 @@
         <v>15.6</v>
       </c>
       <c r="N20" s="1">
-        <v>0</v>
+        <v>36.84683321106351</v>
       </c>
       <c r="O20" t="s">
         <v>35</v>
@@ -20212,7 +20212,7 @@
         <v>317.1</v>
       </c>
       <c r="N21" s="1">
-        <v>0</v>
+        <v>39.89348983754204</v>
       </c>
       <c r="O21" t="s">
         <v>35</v>
@@ -20274,7 +20274,7 @@
         <v>79.19999999999999</v>
       </c>
       <c r="N22" s="1">
-        <v>0</v>
+        <v>39.97390454866906</v>
       </c>
       <c r="O22" t="s">
         <v>36</v>
@@ -20336,7 +20336,7 @@
         <v>175.7</v>
       </c>
       <c r="N23" s="1">
-        <v>0</v>
+        <v>23.98791767505791</v>
       </c>
       <c r="O23" t="s">
         <v>36</v>
@@ -20395,7 +20395,7 @@
         <v>703.8000000000001</v>
       </c>
       <c r="N24" s="1">
-        <v>0</v>
+        <v>57.52353890923705</v>
       </c>
       <c r="O24" t="s">
         <v>36</v>
@@ -20454,7 +20454,7 @@
         <v>35</v>
       </c>
       <c r="N25" s="1">
-        <v>0</v>
+        <v>14.70392847993301</v>
       </c>
       <c r="O25" t="s">
         <v>36</v>
@@ -20516,7 +20516,7 @@
         <v>490</v>
       </c>
       <c r="N26" s="1">
-        <v>0</v>
+        <v>42.73331147173693</v>
       </c>
       <c r="O26" t="s">
         <v>36</v>
@@ -20578,7 +20578,7 @@
         <v>2.4</v>
       </c>
       <c r="N27" s="1">
-        <v>0</v>
+        <v>15.18058663539603</v>
       </c>
       <c r="O27" t="s">
         <v>244</v>
@@ -20640,7 +20640,7 @@
         <v>7.6</v>
       </c>
       <c r="N28" s="1">
-        <v>0</v>
+        <v>15.96951254840345</v>
       </c>
       <c r="O28" t="s">
         <v>35</v>
@@ -20699,7 +20699,7 @@
         <v>22.4</v>
       </c>
       <c r="N29" s="1">
-        <v>0</v>
+        <v>52.56865584596185</v>
       </c>
       <c r="O29" t="s">
         <v>245</v>
@@ -20758,7 +20758,7 @@
         <v>3513</v>
       </c>
       <c r="N30" s="1">
-        <v>0</v>
+        <v>62.32890934486505</v>
       </c>
       <c r="O30" t="s">
         <v>244</v>
@@ -20820,7 +20820,7 @@
         <v>51.2</v>
       </c>
       <c r="N31" s="1">
-        <v>0</v>
+        <v>24.46215824850296</v>
       </c>
       <c r="O31" t="s">
         <v>36</v>
@@ -20882,7 +20882,7 @@
         <v>7.5</v>
       </c>
       <c r="N32" s="1">
-        <v>0</v>
+        <v>12.15260944481739</v>
       </c>
       <c r="O32" t="s">
         <v>35</v>
@@ -20944,7 +20944,7 @@
         <v>155.4</v>
       </c>
       <c r="N33" s="1">
-        <v>0</v>
+        <v>8.035449173674619</v>
       </c>
       <c r="O33" t="s">
         <v>36</v>
@@ -21006,7 +21006,7 @@
         <v>33</v>
       </c>
       <c r="N34" s="1">
-        <v>0</v>
+        <v>10.53226151884099</v>
       </c>
       <c r="O34" t="s">
         <v>35</v>
@@ -21068,7 +21068,7 @@
         <v>524</v>
       </c>
       <c r="N35" s="1">
-        <v>0</v>
+        <v>72.49981043935509</v>
       </c>
       <c r="O35" t="s">
         <v>35</v>
@@ -21130,7 +21130,7 @@
         <v>161.1</v>
       </c>
       <c r="N36" s="1">
-        <v>0</v>
+        <v>22.50712780800693</v>
       </c>
       <c r="O36" t="s">
         <v>36</v>
@@ -21192,7 +21192,7 @@
         <v>23.6</v>
       </c>
       <c r="N37" s="1">
-        <v>0</v>
+        <v>10.1393048335376</v>
       </c>
       <c r="O37" t="s">
         <v>35</v>
@@ -21251,7 +21251,7 @@
         <v>1</v>
       </c>
       <c r="N38" s="1">
-        <v>0</v>
+        <v>6.011831419047602</v>
       </c>
       <c r="O38" t="s">
         <v>35</v>
@@ -21310,7 +21310,7 @@
         <v>42.4</v>
       </c>
       <c r="N39" s="1">
-        <v>0</v>
+        <v>8.35126428294145</v>
       </c>
       <c r="O39" t="s">
         <v>245</v>
@@ -21366,7 +21366,7 @@
         <v>22.8</v>
       </c>
       <c r="N40" s="1">
-        <v>0</v>
+        <v>12.09351633128016</v>
       </c>
       <c r="O40" t="s">
         <v>36</v>
@@ -21425,7 +21425,7 @@
         <v>746</v>
       </c>
       <c r="N41" s="1">
-        <v>0</v>
+        <v>39.63622270594832</v>
       </c>
       <c r="O41" t="s">
         <v>36</v>
@@ -21487,7 +21487,7 @@
         <v>205.2</v>
       </c>
       <c r="N42" s="1">
-        <v>0</v>
+        <v>18.58576019079173</v>
       </c>
       <c r="O42" t="s">
         <v>36</v>
@@ -21546,7 +21546,7 @@
         <v>9.4</v>
       </c>
       <c r="N43" s="1">
-        <v>0</v>
+        <v>10.31192652085174</v>
       </c>
       <c r="O43" t="s">
         <v>244</v>
@@ -21608,7 +21608,7 @@
         <v>4.5</v>
       </c>
       <c r="N44" s="1">
-        <v>0</v>
+        <v>4.698010824388477</v>
       </c>
       <c r="O44" t="s">
         <v>36</v>
@@ -21667,7 +21667,7 @@
         <v>11</v>
       </c>
       <c r="N45" s="1">
-        <v>0</v>
+        <v>4.877372865551081</v>
       </c>
       <c r="O45" t="s">
         <v>35</v>
@@ -21729,7 +21729,7 @@
         <v>1700</v>
       </c>
       <c r="N46" s="1">
-        <v>0</v>
+        <v>56.90917102504978</v>
       </c>
       <c r="O46" t="s">
         <v>246</v>
@@ -21791,7 +21791,7 @@
         <v>378.2</v>
       </c>
       <c r="N47" s="1">
-        <v>0</v>
+        <v>4.670137916513519</v>
       </c>
       <c r="O47" t="s">
         <v>36</v>
@@ -21850,7 +21850,7 @@
         <v>12.5</v>
       </c>
       <c r="N48" s="1">
-        <v>0</v>
+        <v>10.72850944556727</v>
       </c>
       <c r="O48" t="s">
         <v>36</v>
@@ -21909,7 +21909,7 @@
         <v>135.2</v>
       </c>
       <c r="N49" s="1">
-        <v>0</v>
+        <v>7.432917817756545</v>
       </c>
       <c r="O49" t="s">
         <v>36</v>
@@ -21971,7 +21971,7 @@
         <v>33.59999999999999</v>
       </c>
       <c r="N50" s="1">
-        <v>0</v>
+        <v>3.373463696754393</v>
       </c>
       <c r="O50" t="s">
         <v>36</v>
@@ -22030,7 +22030,7 @@
         <v>6</v>
       </c>
       <c r="N51" s="1">
-        <v>0</v>
+        <v>4.268528491562228</v>
       </c>
       <c r="O51" t="s">
         <v>36</v>
@@ -22089,7 +22089,7 @@
         <v>81.89999999999999</v>
       </c>
       <c r="N52" s="1">
-        <v>0</v>
+        <v>20.19270496073999</v>
       </c>
       <c r="O52" t="s">
         <v>36</v>
@@ -22148,7 +22148,7 @@
         <v>483</v>
       </c>
       <c r="N53" s="1">
-        <v>0</v>
+        <v>15.77784856608914</v>
       </c>
       <c r="O53" t="s">
         <v>35</v>
@@ -22210,7 +22210,7 @@
         <v>27</v>
       </c>
       <c r="N54" s="1">
-        <v>0</v>
+        <v>8.411512027490273</v>
       </c>
       <c r="O54" t="s">
         <v>245</v>
@@ -22269,7 +22269,7 @@
         <v>1.3</v>
       </c>
       <c r="N55" s="1">
-        <v>0</v>
+        <v>7.411073055449902</v>
       </c>
       <c r="O55" t="s">
         <v>245</v>
@@ -22328,7 +22328,7 @@
         <v>3.8</v>
       </c>
       <c r="N56" s="1">
-        <v>0</v>
+        <v>7.53578155291019</v>
       </c>
       <c r="O56" t="s">
         <v>35</v>
@@ -22387,7 +22387,7 @@
         <v>1.2</v>
       </c>
       <c r="N57" s="1">
-        <v>0</v>
+        <v>4.930886360942001</v>
       </c>
       <c r="O57" t="s">
         <v>35</v>
@@ -22449,7 +22449,7 @@
         <v>4.4</v>
       </c>
       <c r="N58" s="1">
-        <v>0</v>
+        <v>4.096231117553382</v>
       </c>
       <c r="O58" t="s">
         <v>35</v>
@@ -22511,7 +22511,7 @@
         <v>17</v>
       </c>
       <c r="N59" s="1">
-        <v>0</v>
+        <v>3.688252125541506</v>
       </c>
       <c r="O59" t="s">
         <v>36</v>
@@ -22573,7 +22573,7 @@
         <v>16.2</v>
       </c>
       <c r="N60" s="1">
-        <v>0</v>
+        <v>1.730368188512285</v>
       </c>
       <c r="O60" t="s">
         <v>36</v>
@@ -22629,7 +22629,7 @@
         <v>14.1</v>
       </c>
       <c r="N61" s="1">
-        <v>0</v>
+        <v>8.828634627211466</v>
       </c>
       <c r="O61" t="s">
         <v>243</v>
@@ -22691,7 +22691,7 @@
         <v>48</v>
       </c>
       <c r="N62" s="1">
-        <v>0</v>
+        <v>4.381960778505825</v>
       </c>
       <c r="O62" t="s">
         <v>36</v>
@@ -22753,7 +22753,7 @@
         <v>119.2</v>
       </c>
       <c r="N63" s="1">
-        <v>0</v>
+        <v>25.33756685174794</v>
       </c>
       <c r="O63" t="s">
         <v>36</v>
@@ -22895,7 +22895,7 @@
         <v>4723</v>
       </c>
       <c r="N2" s="1">
-        <v>0</v>
+        <v>95.28846510115214</v>
       </c>
       <c r="O2" t="s">
         <v>244</v>
@@ -22957,7 +22957,7 @@
         <v>3843</v>
       </c>
       <c r="N3" s="1">
-        <v>0</v>
+        <v>525.6239049259281</v>
       </c>
       <c r="O3" t="s">
         <v>244</v>
@@ -23019,7 +23019,7 @@
         <v>3513</v>
       </c>
       <c r="N4" s="1">
-        <v>0</v>
+        <v>62.32890934486505</v>
       </c>
       <c r="O4" t="s">
         <v>244</v>
@@ -23081,7 +23081,7 @@
         <v>3417</v>
       </c>
       <c r="N5" s="1">
-        <v>0</v>
+        <v>42.84307302105591</v>
       </c>
       <c r="O5" t="s">
         <v>35</v>
@@ -23143,7 +23143,7 @@
         <v>3087</v>
       </c>
       <c r="N6" s="1">
-        <v>0</v>
+        <v>79.09953304865576</v>
       </c>
       <c r="O6" t="s">
         <v>36</v>
@@ -23205,7 +23205,7 @@
         <v>2824</v>
       </c>
       <c r="N7" s="1">
-        <v>0</v>
+        <v>82.11893633265019</v>
       </c>
       <c r="O7" t="s">
         <v>35</v>
@@ -23267,7 +23267,7 @@
         <v>2138.4</v>
       </c>
       <c r="N8" s="1">
-        <v>0</v>
+        <v>33.7807946476311</v>
       </c>
       <c r="O8" t="s">
         <v>243</v>
@@ -23329,7 +23329,7 @@
         <v>2028</v>
       </c>
       <c r="N9" s="1">
-        <v>0</v>
+        <v>27.06582596638111</v>
       </c>
       <c r="O9" t="s">
         <v>35</v>
@@ -23391,7 +23391,7 @@
         <v>1700</v>
       </c>
       <c r="N10" s="1">
-        <v>0</v>
+        <v>56.90917102504978</v>
       </c>
       <c r="O10" t="s">
         <v>246</v>
@@ -23453,7 +23453,7 @@
         <v>1598</v>
       </c>
       <c r="N11" s="1">
-        <v>0</v>
+        <v>94.4718123952869</v>
       </c>
       <c r="O11" t="s">
         <v>35</v>
@@ -23515,7 +23515,7 @@
         <v>1445</v>
       </c>
       <c r="N12" s="1">
-        <v>0</v>
+        <v>33.63271709201708</v>
       </c>
       <c r="O12" t="s">
         <v>35</v>
@@ -23577,7 +23577,7 @@
         <v>1406.7</v>
       </c>
       <c r="N13" s="1">
-        <v>0</v>
+        <v>6861.283954608292</v>
       </c>
       <c r="O13" t="s">
         <v>35</v>
@@ -23639,7 +23639,7 @@
         <v>1242</v>
       </c>
       <c r="N14" s="1">
-        <v>0</v>
+        <v>49.81580339270992</v>
       </c>
       <c r="O14" t="s">
         <v>36</v>
@@ -23698,7 +23698,7 @@
         <v>1148</v>
       </c>
       <c r="N15" s="1">
-        <v>0</v>
+        <v>69.19683453679401</v>
       </c>
       <c r="O15" t="s">
         <v>35</v>
@@ -23760,7 +23760,7 @@
         <v>961.6</v>
       </c>
       <c r="N16" s="1">
-        <v>0</v>
+        <v>5.119157635505013</v>
       </c>
       <c r="O16" t="s">
         <v>35</v>
@@ -23819,7 +23819,7 @@
         <v>921.6</v>
       </c>
       <c r="N17" s="1">
-        <v>0</v>
+        <v>84.72706744014472</v>
       </c>
       <c r="O17" t="s">
         <v>36</v>
@@ -23878,7 +23878,7 @@
         <v>872</v>
       </c>
       <c r="N18" s="1">
-        <v>0</v>
+        <v>17.93764447325695</v>
       </c>
       <c r="O18" t="s">
         <v>36</v>
@@ -23937,7 +23937,7 @@
         <v>853.6</v>
       </c>
       <c r="N19" s="1">
-        <v>0</v>
+        <v>8.205439441347828</v>
       </c>
       <c r="O19" t="s">
         <v>36</v>
@@ -23999,7 +23999,7 @@
         <v>818</v>
       </c>
       <c r="N20" s="1">
-        <v>0</v>
+        <v>74.49584127135387</v>
       </c>
       <c r="O20" t="s">
         <v>36</v>
@@ -24058,7 +24058,7 @@
         <v>757.4</v>
       </c>
       <c r="N21" s="1">
-        <v>0</v>
+        <v>42.1406087983756</v>
       </c>
       <c r="O21" t="s">
         <v>36</v>
@@ -24117,7 +24117,7 @@
         <v>746</v>
       </c>
       <c r="N22" s="1">
-        <v>0</v>
+        <v>39.63622270594832</v>
       </c>
       <c r="O22" t="s">
         <v>36</v>
@@ -24179,7 +24179,7 @@
         <v>703.8000000000001</v>
       </c>
       <c r="N23" s="1">
-        <v>0</v>
+        <v>57.52353890923705</v>
       </c>
       <c r="O23" t="s">
         <v>36</v>
@@ -24238,7 +24238,7 @@
         <v>693</v>
       </c>
       <c r="N24" s="1">
-        <v>0</v>
+        <v>149.8194801835526</v>
       </c>
       <c r="O24" t="s">
         <v>35</v>
@@ -24300,7 +24300,7 @@
         <v>687.6</v>
       </c>
       <c r="N25" s="1">
-        <v>0</v>
+        <v>250.37449587335</v>
       </c>
       <c r="O25" t="s">
         <v>244</v>
@@ -24362,7 +24362,7 @@
         <v>686.6999999999999</v>
       </c>
       <c r="N26" s="1">
-        <v>0</v>
+        <v>15.83093927041445</v>
       </c>
       <c r="O26" t="s">
         <v>36</v>
@@ -24424,7 +24424,7 @@
         <v>648</v>
       </c>
       <c r="N27" s="1">
-        <v>0</v>
+        <v>307.105540245145</v>
       </c>
       <c r="O27" t="s">
         <v>35</v>
@@ -24486,7 +24486,7 @@
         <v>609.3000000000001</v>
       </c>
       <c r="N28" s="1">
-        <v>0</v>
+        <v>471.1258262275985</v>
       </c>
       <c r="O28" t="s">
         <v>35</v>
@@ -24548,7 +24548,7 @@
         <v>559.2</v>
       </c>
       <c r="N29" s="1">
-        <v>0</v>
+        <v>516.9986322673582</v>
       </c>
       <c r="O29" t="s">
         <v>35</v>
@@ -24610,7 +24610,7 @@
         <v>551.6999999999999</v>
       </c>
       <c r="N30" s="1">
-        <v>0</v>
+        <v>17.88233177571537</v>
       </c>
       <c r="O30" t="s">
         <v>35</v>
@@ -24672,7 +24672,7 @@
         <v>524</v>
       </c>
       <c r="N31" s="1">
-        <v>0</v>
+        <v>72.49981043935509</v>
       </c>
       <c r="O31" t="s">
         <v>35</v>
@@ -24734,7 +24734,7 @@
         <v>500.4</v>
       </c>
       <c r="N32" s="1">
-        <v>0</v>
+        <v>21.41117833339402</v>
       </c>
       <c r="O32" t="s">
         <v>36</v>
@@ -24796,7 +24796,7 @@
         <v>490</v>
       </c>
       <c r="N33" s="1">
-        <v>0</v>
+        <v>42.73331147173693</v>
       </c>
       <c r="O33" t="s">
         <v>36</v>
@@ -24858,7 +24858,7 @@
         <v>483</v>
       </c>
       <c r="N34" s="1">
-        <v>0</v>
+        <v>15.77784856608914</v>
       </c>
       <c r="O34" t="s">
         <v>35</v>
@@ -24920,7 +24920,7 @@
         <v>469.8</v>
       </c>
       <c r="N35" s="1">
-        <v>0</v>
+        <v>101.8869347047059</v>
       </c>
       <c r="O35" t="s">
         <v>36</v>
@@ -24982,7 +24982,7 @@
         <v>410.4</v>
       </c>
       <c r="N36" s="1">
-        <v>0</v>
+        <v>222.878410285862</v>
       </c>
       <c r="O36" t="s">
         <v>35</v>
@@ -25044,7 +25044,7 @@
         <v>408</v>
       </c>
       <c r="N37" s="1">
-        <v>0</v>
+        <v>14.12382153621653</v>
       </c>
       <c r="O37" t="s">
         <v>246</v>
@@ -25106,7 +25106,7 @@
         <v>378.2</v>
       </c>
       <c r="N38" s="1">
-        <v>0</v>
+        <v>4.670137916513519</v>
       </c>
       <c r="O38" t="s">
         <v>36</v>
@@ -25165,7 +25165,7 @@
         <v>370</v>
       </c>
       <c r="N39" s="1">
-        <v>0</v>
+        <v>30.63158816206036</v>
       </c>
       <c r="O39" t="s">
         <v>244</v>
@@ -25227,7 +25227,7 @@
         <v>365.6</v>
       </c>
       <c r="N40" s="1">
-        <v>0</v>
+        <v>386.1732049325275</v>
       </c>
       <c r="O40" t="s">
         <v>35</v>
@@ -25289,7 +25289,7 @@
         <v>351.2</v>
       </c>
       <c r="N41" s="1">
-        <v>0</v>
+        <v>19.31609516060931</v>
       </c>
       <c r="O41" t="s">
         <v>36</v>
@@ -25351,7 +25351,7 @@
         <v>350</v>
       </c>
       <c r="N42" s="1">
-        <v>0</v>
+        <v>7.644018814864816</v>
       </c>
       <c r="O42" t="s">
         <v>35</v>
@@ -25413,7 +25413,7 @@
         <v>317.1</v>
       </c>
       <c r="N43" s="1">
-        <v>0</v>
+        <v>39.89348983754204</v>
       </c>
       <c r="O43" t="s">
         <v>35</v>
@@ -25475,7 +25475,7 @@
         <v>280</v>
       </c>
       <c r="N44" s="1">
-        <v>0</v>
+        <v>20.28554497550737</v>
       </c>
       <c r="O44" t="s">
         <v>243</v>
@@ -25537,7 +25537,7 @@
         <v>272.8</v>
       </c>
       <c r="N45" s="1">
-        <v>0</v>
+        <v>104.6321499926035</v>
       </c>
       <c r="O45" t="s">
         <v>35</v>
@@ -25599,7 +25599,7 @@
         <v>265.5</v>
       </c>
       <c r="N46" s="1">
-        <v>0</v>
+        <v>240.3390775357394</v>
       </c>
       <c r="O46" t="s">
         <v>35</v>
@@ -25661,7 +25661,7 @@
         <v>240.1</v>
       </c>
       <c r="N47" s="1">
-        <v>0</v>
+        <v>7.778839321565147</v>
       </c>
       <c r="O47" t="s">
         <v>36</v>
@@ -25723,7 +25723,7 @@
         <v>211.2</v>
       </c>
       <c r="N48" s="1">
-        <v>0</v>
+        <v>74.20554420607192</v>
       </c>
       <c r="O48" t="s">
         <v>36</v>
@@ -25782,7 +25782,7 @@
         <v>205.2</v>
       </c>
       <c r="N49" s="1">
-        <v>0</v>
+        <v>18.58576019079173</v>
       </c>
       <c r="O49" t="s">
         <v>36</v>
@@ -25841,7 +25841,7 @@
         <v>201.6</v>
       </c>
       <c r="N50" s="1">
-        <v>0</v>
+        <v>387.2525226207051</v>
       </c>
       <c r="O50" t="s">
         <v>36</v>
@@ -25900,7 +25900,7 @@
         <v>190.4</v>
       </c>
       <c r="N51" s="1">
-        <v>0</v>
+        <v>5.083461083498125</v>
       </c>
       <c r="O51" t="s">
         <v>36</v>
@@ -25962,7 +25962,7 @@
         <v>189.6</v>
       </c>
       <c r="N52" s="1">
-        <v>0</v>
+        <v>40.02223498224424</v>
       </c>
       <c r="O52" t="s">
         <v>35</v>
@@ -26024,7 +26024,7 @@
         <v>185.6</v>
       </c>
       <c r="N53" s="1">
-        <v>0</v>
+        <v>3.187988318213764</v>
       </c>
       <c r="O53" t="s">
         <v>36</v>
@@ -26086,7 +26086,7 @@
         <v>177.6</v>
       </c>
       <c r="N54" s="1">
-        <v>0</v>
+        <v>140.3766571528158</v>
       </c>
       <c r="O54" t="s">
         <v>35</v>
@@ -26148,7 +26148,7 @@
         <v>175.7</v>
       </c>
       <c r="N55" s="1">
-        <v>0</v>
+        <v>23.98791767505791</v>
       </c>
       <c r="O55" t="s">
         <v>36</v>
@@ -26207,7 +26207,7 @@
         <v>161.1</v>
       </c>
       <c r="N56" s="1">
-        <v>0</v>
+        <v>22.50712780800693</v>
       </c>
       <c r="O56" t="s">
         <v>36</v>
@@ -26269,7 +26269,7 @@
         <v>155.4</v>
       </c>
       <c r="N57" s="1">
-        <v>0</v>
+        <v>8.035449173674619</v>
       </c>
       <c r="O57" t="s">
         <v>36</v>
@@ -26331,7 +26331,7 @@
         <v>148</v>
       </c>
       <c r="N58" s="1">
-        <v>0</v>
+        <v>13.42953312578718</v>
       </c>
       <c r="O58" t="s">
         <v>35</v>
@@ -26393,7 +26393,7 @@
         <v>144.8</v>
       </c>
       <c r="N59" s="1">
-        <v>0</v>
+        <v>208.3982879751641</v>
       </c>
       <c r="O59" t="s">
         <v>36</v>
@@ -26452,7 +26452,7 @@
         <v>143</v>
       </c>
       <c r="N60" s="1">
-        <v>0</v>
+        <v>6.719535260243862</v>
       </c>
       <c r="O60" t="s">
         <v>36</v>
@@ -26511,7 +26511,7 @@
         <v>142.2</v>
       </c>
       <c r="N61" s="1">
-        <v>0</v>
+        <v>83.42707445865703</v>
       </c>
       <c r="O61" t="s">
         <v>35</v>
@@ -26573,7 +26573,7 @@
         <v>136.8</v>
       </c>
       <c r="N62" s="1">
-        <v>0</v>
+        <v>234.3091776640756</v>
       </c>
       <c r="O62" t="s">
         <v>36</v>
@@ -26635,7 +26635,7 @@
         <v>135.2</v>
       </c>
       <c r="N63" s="1">
-        <v>0</v>
+        <v>7.432917817756545</v>
       </c>
       <c r="O63" t="s">
         <v>36</v>
@@ -26697,7 +26697,7 @@
         <v>133.2</v>
       </c>
       <c r="N64" s="1">
-        <v>0</v>
+        <v>4.490634878002823</v>
       </c>
       <c r="O64" t="s">
         <v>36</v>
@@ -26759,7 +26759,7 @@
         <v>132.5</v>
       </c>
       <c r="N65" s="1">
-        <v>0</v>
+        <v>3.900953436672769</v>
       </c>
       <c r="O65" t="s">
         <v>35</v>
@@ -26821,7 +26821,7 @@
         <v>132</v>
       </c>
       <c r="N66" s="1">
-        <v>0</v>
+        <v>73.18186678178051</v>
       </c>
       <c r="O66" t="s">
         <v>35</v>
@@ -26883,7 +26883,7 @@
         <v>127.2</v>
       </c>
       <c r="N67" s="1">
-        <v>0</v>
+        <v>207.8292216279649</v>
       </c>
       <c r="O67" t="s">
         <v>35</v>
@@ -26945,7 +26945,7 @@
         <v>119.2</v>
       </c>
       <c r="N68" s="1">
-        <v>0</v>
+        <v>25.33756685174794</v>
       </c>
       <c r="O68" t="s">
         <v>36</v>
@@ -27004,7 +27004,7 @@
         <v>118</v>
       </c>
       <c r="N69" s="1">
-        <v>0</v>
+        <v>58.69041087703511</v>
       </c>
       <c r="O69" t="s">
         <v>35</v>
@@ -27066,7 +27066,7 @@
         <v>117</v>
       </c>
       <c r="N70" s="1">
-        <v>0</v>
+        <v>3.884940769227031</v>
       </c>
       <c r="O70" t="s">
         <v>36</v>
@@ -27122,7 +27122,7 @@
         <v>116</v>
       </c>
       <c r="N71" s="1">
-        <v>0</v>
+        <v>90.6630193990094</v>
       </c>
       <c r="O71" t="s">
         <v>36</v>
@@ -27184,7 +27184,7 @@
         <v>115.2</v>
       </c>
       <c r="N72" s="1">
-        <v>0</v>
+        <v>922.4202957440928</v>
       </c>
       <c r="O72" t="s">
         <v>35</v>
@@ -27246,7 +27246,7 @@
         <v>108</v>
       </c>
       <c r="N73" s="1">
-        <v>0</v>
+        <v>36.09020464778688</v>
       </c>
       <c r="O73" t="s">
         <v>35</v>
@@ -27308,7 +27308,7 @@
         <v>94.5</v>
       </c>
       <c r="N74" s="1">
-        <v>0</v>
+        <v>1.360706788473817</v>
       </c>
       <c r="O74" t="s">
         <v>278</v>
@@ -27367,7 +27367,7 @@
         <v>93.90000000000001</v>
       </c>
       <c r="N75" s="1">
-        <v>0</v>
+        <v>3.036991043139647</v>
       </c>
       <c r="O75" t="s">
         <v>36</v>
@@ -27426,7 +27426,7 @@
         <v>89.60000000000001</v>
       </c>
       <c r="N76" s="1">
-        <v>0</v>
+        <v>248.4356548388555</v>
       </c>
       <c r="O76" t="s">
         <v>35</v>
@@ -27488,7 +27488,7 @@
         <v>81.89999999999999</v>
       </c>
       <c r="N77" s="1">
-        <v>0</v>
+        <v>20.19270496073999</v>
       </c>
       <c r="O77" t="s">
         <v>36</v>
@@ -27547,7 +27547,7 @@
         <v>80.2</v>
       </c>
       <c r="N78" s="1">
-        <v>0</v>
+        <v>2.591989037920724</v>
       </c>
       <c r="O78" t="s">
         <v>243</v>
@@ -27609,7 +27609,7 @@
         <v>79.19999999999999</v>
       </c>
       <c r="N79" s="1">
-        <v>0</v>
+        <v>39.97390454866906</v>
       </c>
       <c r="O79" t="s">
         <v>36</v>
@@ -27671,7 +27671,7 @@
         <v>74.40000000000001</v>
       </c>
       <c r="N80" s="1">
-        <v>0</v>
+        <v>4.432866838487374</v>
       </c>
       <c r="O80" t="s">
         <v>35</v>
@@ -27733,7 +27733,7 @@
         <v>74.09999999999999</v>
       </c>
       <c r="N81" s="1">
-        <v>0</v>
+        <v>5.763286156288465</v>
       </c>
       <c r="O81" t="s">
         <v>35</v>
@@ -27795,7 +27795,7 @@
         <v>65.10000000000001</v>
       </c>
       <c r="N82" s="1">
-        <v>0</v>
+        <v>18.23429176317842</v>
       </c>
       <c r="O82" t="s">
         <v>36</v>
@@ -27854,7 +27854,7 @@
         <v>65</v>
       </c>
       <c r="N83" s="1">
-        <v>0</v>
+        <v>5.036083056079515</v>
       </c>
       <c r="O83" t="s">
         <v>35</v>
@@ -27916,7 +27916,7 @@
         <v>55.2</v>
       </c>
       <c r="N84" s="1">
-        <v>0</v>
+        <v>3.253820945677159</v>
       </c>
       <c r="O84" t="s">
         <v>36</v>
@@ -27972,7 +27972,7 @@
         <v>52</v>
       </c>
       <c r="N85" s="1">
-        <v>0</v>
+        <v>4.224273047748467</v>
       </c>
       <c r="O85" t="s">
         <v>244</v>
@@ -28034,7 +28034,7 @@
         <v>51.2</v>
       </c>
       <c r="N86" s="1">
-        <v>0</v>
+        <v>24.46215824850296</v>
       </c>
       <c r="O86" t="s">
         <v>36</v>
@@ -28096,7 +28096,7 @@
         <v>50.40000000000001</v>
       </c>
       <c r="N87" s="1">
-        <v>0</v>
+        <v>14.4821181545651</v>
       </c>
       <c r="O87" t="s">
         <v>245</v>
@@ -28155,7 +28155,7 @@
         <v>50.4</v>
       </c>
       <c r="N88" s="1">
-        <v>0</v>
+        <v>128.4966051306644</v>
       </c>
       <c r="O88" t="s">
         <v>245</v>
@@ -28214,7 +28214,7 @@
         <v>48</v>
       </c>
       <c r="N89" s="1">
-        <v>0</v>
+        <v>4.381960778505825</v>
       </c>
       <c r="O89" t="s">
         <v>36</v>
@@ -28276,7 +28276,7 @@
         <v>42.4</v>
       </c>
       <c r="N90" s="1">
-        <v>0</v>
+        <v>8.35126428294145</v>
       </c>
       <c r="O90" t="s">
         <v>245</v>
@@ -28332,7 +28332,7 @@
         <v>37.6</v>
       </c>
       <c r="N91" s="1">
-        <v>0</v>
+        <v>333.5745409603368</v>
       </c>
       <c r="O91" t="s">
         <v>243</v>
@@ -28394,7 +28394,7 @@
         <v>35</v>
       </c>
       <c r="N92" s="1">
-        <v>0</v>
+        <v>14.70392847993301</v>
       </c>
       <c r="O92" t="s">
         <v>36</v>
@@ -28456,7 +28456,7 @@
         <v>33.59999999999999</v>
       </c>
       <c r="N93" s="1">
-        <v>0</v>
+        <v>3.373463696754393</v>
       </c>
       <c r="O93" t="s">
         <v>36</v>
@@ -28515,7 +28515,7 @@
         <v>33</v>
       </c>
       <c r="N94" s="1">
-        <v>0</v>
+        <v>10.53226151884099</v>
       </c>
       <c r="O94" t="s">
         <v>35</v>
@@ -28577,7 +28577,7 @@
         <v>33</v>
       </c>
       <c r="N95" s="1">
-        <v>0</v>
+        <v>35.80317334918507</v>
       </c>
       <c r="O95" t="s">
         <v>35</v>
@@ -28639,7 +28639,7 @@
         <v>32.09999999999999</v>
       </c>
       <c r="N96" s="1">
-        <v>0</v>
+        <v>2.388843150352038</v>
       </c>
       <c r="O96" t="s">
         <v>35</v>
@@ -28698,7 +28698,7 @@
         <v>29.2</v>
       </c>
       <c r="N97" s="1">
-        <v>0</v>
+        <v>32.7958730628951</v>
       </c>
       <c r="O97" t="s">
         <v>35</v>
@@ -28760,7 +28760,7 @@
         <v>28</v>
       </c>
       <c r="N98" s="1">
-        <v>0</v>
+        <v>4.410947131822462</v>
       </c>
       <c r="O98" t="s">
         <v>36</v>
@@ -28816,7 +28816,7 @@
         <v>27</v>
       </c>
       <c r="N99" s="1">
-        <v>0</v>
+        <v>8.411512027490273</v>
       </c>
       <c r="O99" t="s">
         <v>245</v>
@@ -28875,7 +28875,7 @@
         <v>26.4</v>
       </c>
       <c r="N100" s="1">
-        <v>0</v>
+        <v>9.854643729556518</v>
       </c>
       <c r="O100" t="s">
         <v>245</v>
@@ -28934,7 +28934,7 @@
         <v>24</v>
       </c>
       <c r="N101" s="1">
-        <v>0</v>
+        <v>5.649213015993937</v>
       </c>
       <c r="O101" t="s">
         <v>35</v>

</xml_diff>